<commit_message>
update pglm and ort supp tables
</commit_message>
<xml_diff>
--- a/results/Supplementary_Table_6_OddsRatioTest_interesting_hits.xlsx
+++ b/results/Supplementary_Table_6_OddsRatioTest_interesting_hits.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,76 +425,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>HOG</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Occupancy</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Log odds ratio of loss</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Log odds ratio of duplication</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>LOR outside permuted avg thresholds</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P-value, loss more likely in orb-weavers</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>P-value, loss more likely in non-orb-weavers</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>P-value, duplication more likely in orb-weavers</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>P-value, duplication more likely in non-orb-weavers</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>U. diversus gene ID</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>U. diversus GO terms</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>U. diversus gene description</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>P. tepidariorum best BLAST hit for the HOG</t>
         </is>
@@ -496,17 +508,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>1.611461457641113</v>
+        <v>1.9468698070612</v>
       </c>
       <c r="E2" t="n">
-        <v>-1.686717262108546</v>
+        <v>-1.544702271122541</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -514,16 +526,16 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.108</v>
+        <v>0.0165</v>
       </c>
       <c r="H2" t="n">
-        <v>0.892</v>
+        <v>0.9835</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9500999999999999</v>
+        <v>0.9383</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0499</v>
+        <v>0.0617</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -549,22 +561,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>N5.HOG0016850</t>
+          <t>N5.HOG0014159</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.470831893915742</v>
+        <v>0.1695128339342781</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.6175850486563819</v>
+        <v>2.093719810042682</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -572,35 +584,35 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.9868</v>
+        <v>0.3622</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0132</v>
+        <v>0.6378</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6464</v>
+        <v>0.0394</v>
       </c>
       <c r="J3" t="n">
-        <v>0.3534</v>
+        <v>0.9606</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>129234104</t>
+          <t>129217691</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>GO:0006468 [Name: protein phosphorylation]; GO:0004692 [Name: cGMP-dependent protein kinase activity]; GO:0005524 [Name: ATP binding]</t>
+          <t>GO:0005109 [Name: frizzled binding]; GO:0005576 [Name: extracellular region]; GO:0007275 [Name: multicellular organism development]; GO:0005615 [Name: extracellular space]; GO:0005125 [Name: cytokine activity]; GO:0045165 [Name: cell fate commitment]; GO:0060070 [Name: canonical Wnt signaling pathway]; GO:0030182 [Name: neuron differentiation]</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>cGMP-dependent protein kinase, isozyme 2 forms cD4/T1/T3A/T3B-like</t>
+          <t>protein Wnt-16-like</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>cGMP-dependent protein kinase 1 isoform X4</t>
+          <t>protein Wnt-16-like precursor</t>
         </is>
       </c>
     </row>
@@ -619,10 +631,10 @@
         <v>84</v>
       </c>
       <c r="D4" t="n">
-        <v>-1.626481296043397</v>
+        <v>-1.480659154768488</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7655609713165419</v>
+        <v>0.3954992145445163</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -630,16 +642,16 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.9864000000000001</v>
+        <v>0.9706</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0136</v>
+        <v>0.0294</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1582</v>
+        <v>0.3609</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8418</v>
+        <v>0.6391</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -665,7 +677,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>N5.HOG0019920</t>
+          <t>N5.HOG0022330</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -674,172 +686,172 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="D5" t="n">
-        <v>-3.668798878026179</v>
+        <v>-2.722522137196489</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9254294632427672</v>
+        <v>2.1413448640213</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.9766</v>
+        <v>0.9938</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0234</v>
+        <v>0.0062</v>
       </c>
       <c r="I5" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.0579</v>
       </c>
       <c r="J5" t="n">
-        <v>0.9048</v>
+        <v>0.9421</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>129222487</t>
+          <t>129217545</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>GO:0005515 [Name: protein binding]; GO:0007052 [Name: mitotic spindle organization]; GO:0007346 [Name: regulation of mitotic cell cycle]; GO:0072686 [Name: mitotic spindle]</t>
+          <t>GO:0046777 [Name: protein autophosphorylation]; GO:0005634 [Name: nucleus]; GO:0004712 [Name: protein serine/threonine/tyrosine kinase activity]; GO:0005524 [Name: ATP binding]; GO:0018107 [Name: peptidyl-threonine phosphorylation]; GO:0045893 [Name: positive regulation of transcription, DNA-templated]; GO:0018105 [Name: peptidyl-serine phosphorylation]; GO:0003713 [Name: transcription coactivator activity]; GO:0004674 [Name: protein serine/threonine kinase activity]</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>mitogen-activated protein kinase-binding protein 1-like</t>
+          <t>dual specificity tyrosine-phosphorylation-regulated kinase 1B-like</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>mitogen-activated protein kinase-binding protein 1 isoform X1</t>
+          <t>dual specificity tyrosine-phosphorylation-regulated kinase 1B</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>N5.HOG0022330</t>
+          <t>N5.HOG0024065</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers, duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="D6" t="n">
-        <v>-2.749680139594894</v>
+        <v>-2.850323652297765</v>
       </c>
       <c r="E6" t="n">
-        <v>2.013628138798434</v>
+        <v>2.026190682728394</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes for loss; no for duplication</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.9837</v>
+        <v>0.9583</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0163</v>
+        <v>0.0417</v>
       </c>
       <c r="I6" t="n">
-        <v>0.07190000000000001</v>
+        <v>0.0115</v>
       </c>
       <c r="J6" t="n">
-        <v>0.9281</v>
+        <v>0.9885</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>129217545</t>
+          <t>129218972</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>GO:0046777 [Name: protein autophosphorylation]; GO:0005634 [Name: nucleus]; GO:0004712 [Name: protein serine/threonine/tyrosine kinase activity]; GO:0005524 [Name: ATP binding]; GO:0018107 [Name: peptidyl-threonine phosphorylation]; GO:0045893 [Name: positive regulation of transcription, DNA-templated]; GO:0018105 [Name: peptidyl-serine phosphorylation]; GO:0003713 [Name: transcription coactivator activity]; GO:0004674 [Name: protein serine/threonine kinase activity]</t>
+          <t>GO:0005737 [Name: cytoplasm]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]; GO:0000226 [Name: microtubule cytoskeleton organization]; GO:0035556 [Name: intracellular signal transduction]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0050321 [Name: tau-protein kinase activity]</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>dual specificity tyrosine-phosphorylation-regulated kinase 1B-like</t>
+          <t>uncharacterized LOC129218972</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>dual specificity tyrosine-phosphorylation-regulated kinase 1B</t>
+          <t>uncharacterized protein</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>N5.HOG0024065</t>
+          <t>N5.HOG0027025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers, duplication more likely in orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="D7" t="n">
-        <v>-3.043582781496684</v>
+        <v>0.3724852135764452</v>
       </c>
       <c r="E7" t="n">
-        <v>1.83672402662492</v>
+        <v>1.534842341028485</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Yes for loss; no for duplication</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.9656</v>
+        <v>0.3559</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0344</v>
+        <v>0.6441</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0353</v>
+        <v>0.013</v>
       </c>
       <c r="J7" t="n">
-        <v>0.9647</v>
+        <v>0.987</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>129218972</t>
+          <t>129224223</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>GO:0005737 [Name: cytoplasm]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]; GO:0000226 [Name: microtubule cytoskeleton organization]; GO:0035556 [Name: intracellular signal transduction]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0050321 [Name: tau-protein kinase activity]</t>
+          <t>GO:0005524 [Name: ATP binding]; GO:0005007 [Name: fibroblast growth factor-activated receptor activity]; GO:0033674 [Name: positive regulation of kinase activity]; GO:0006468 [Name: protein phosphorylation]; GO:0008543 [Name: fibroblast growth factor receptor signaling pathway]; GO:0043235 [Name: receptor complex]; GO:0007275 [Name: multicellular organism development]; GO:0016020 [Name: membrane]; GO:0008284 [Name: positive regulation of cell proliferation]</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>uncharacterized LOC129218972</t>
+          <t>fibroblast growth factor receptor 4-like</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>uncharacterized protein</t>
+          <t>fibroblast growth factor receptor 3</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>N5.HOG0024517</t>
+          <t>N5.HOG0027166</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -848,13 +860,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D8" t="n">
-        <v>-2.433674822083392</v>
+        <v>-1.848016277561112</v>
       </c>
       <c r="E8" t="n">
-        <v>1.35317819378956</v>
+        <v>0.649585850409377</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -862,57 +874,57 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.9505</v>
+        <v>0.9571</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0495</v>
+        <v>0.0429</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1818</v>
+        <v>0.0929</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8182</v>
+        <v>0.9071</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>129226511</t>
+          <t>129218261</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>GO:0000287 [Name: magnesium ion binding]; GO:0005524 [Name: ATP binding]; GO:0035556 [Name: intracellular signal transduction]; GO:0006468 [Name: protein phosphorylation]; GO:0004711 [Name: ribosomal protein S6 kinase activity]</t>
+          <t>GO:0004672 [Name: protein kinase activity]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>ribosomal protein S6 kinase 2 beta-like</t>
+          <t>serine/threonine-protein kinase Nek4-like</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>ribosomal protein S6 kinase 2 beta isoform X1</t>
+          <t>uncharacterized protein isoform X2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>N5.HOG0027025</t>
+          <t>N5.HOG0030179</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Duplication more likely in orb-weavers</t>
+          <t>Loss more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2273396449503494</v>
+        <v>2.198879340274023</v>
       </c>
       <c r="E9" t="n">
-        <v>1.901252383982568</v>
+        <v>-0.5104480232027152</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -920,57 +932,57 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.4456</v>
+        <v>0.0017</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5544</v>
+        <v>0.9983</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0125</v>
+        <v>0.7064</v>
       </c>
       <c r="J9" t="n">
-        <v>0.9875</v>
+        <v>0.2936</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>129224223</t>
+          <t>129221278</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>GO:0005524 [Name: ATP binding]; GO:0005007 [Name: fibroblast growth factor-activated receptor activity]; GO:0033674 [Name: positive regulation of kinase activity]; GO:0006468 [Name: protein phosphorylation]; GO:0008543 [Name: fibroblast growth factor receptor signaling pathway]; GO:0043235 [Name: receptor complex]; GO:0007275 [Name: multicellular organism development]; GO:0016020 [Name: membrane]; GO:0008284 [Name: positive regulation of cell proliferation]</t>
+          <t>GO:0005524 [Name: ATP binding]; GO:0007156 [Name: homophilic cell adhesion via plasma membrane adhesion molecules]; GO:0030424 [Name: axon]; GO:0004672 [Name: protein kinase activity]; GO:0006468 [Name: protein phosphorylation]; GO:0007411 [Name: axon guidance]; GO:0070593 [Name: dendrite self-avoidance]; GO:0098632 [Name: protein binding involved in cell-cell adhesion]; GO:0005886 [Name: plasma membrane]</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>fibroblast growth factor receptor 4-like</t>
+          <t>inactive tyrosine-protein kinase 7-like</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>fibroblast growth factor receptor 3</t>
+          <t>inactive tyrosine-protein kinase 7</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>N5.HOG0030179</t>
+          <t>N5.HOG0030685</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Loss more likely in orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="D10" t="n">
-        <v>2.29943126625738</v>
+        <v>-0.5231918341899076</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.641408076212985</v>
+        <v>-1.881225644050893</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -978,289 +990,289 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.0018</v>
+        <v>0.598</v>
       </c>
       <c r="H10" t="n">
-        <v>0.9982</v>
+        <v>0.4019</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7042</v>
+        <v>0.9766</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2958</v>
+        <v>0.0234</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>129221278</t>
+          <t>129227393</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>GO:0005524 [Name: ATP binding]; GO:0007156 [Name: homophilic cell adhesion via plasma membrane adhesion molecules]; GO:0030424 [Name: axon]; GO:0004672 [Name: protein kinase activity]; GO:0006468 [Name: protein phosphorylation]; GO:0007411 [Name: axon guidance]; GO:0070593 [Name: dendrite self-avoidance]; GO:0098632 [Name: protein binding involved in cell-cell adhesion]; GO:0005886 [Name: plasma membrane]</t>
+          <t>GO:0005737 [Name: cytoplasm]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]; GO:0005634 [Name: nucleus]; GO:0030036 [Name: actin cytoskeleton organization]; GO:0005515 [Name: protein binding]</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>inactive tyrosine-protein kinase 7-like</t>
+          <t>LIM domain kinase 1</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>inactive tyrosine-protein kinase 7</t>
+          <t>LIM domain kinase 1 isoform X3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>N5.HOG0030685</t>
+          <t>N5.HOG0030687</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.6551747951999796</v>
+        <v>-3.971010727632098</v>
       </c>
       <c r="E11" t="n">
-        <v>-2.030220553492037</v>
+        <v>-0.466919899779848</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.7274</v>
+        <v>0.9528</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2726</v>
+        <v>0.0472</v>
       </c>
       <c r="I11" t="n">
-        <v>0.9826</v>
+        <v>0.5985</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0174</v>
+        <v>0.4015</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>129227393</t>
+          <t>129233658</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>GO:0005737 [Name: cytoplasm]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]; GO:0005634 [Name: nucleus]; GO:0030036 [Name: actin cytoskeleton organization]; GO:0005515 [Name: protein binding]</t>
+          <t>GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005515 [Name: protein binding]; GO:0005737 [Name: cytoplasm]; GO:0006468 [Name: protein phosphorylation]; GO:0030036 [Name: actin cytoskeleton organization]; GO:0005524 [Name: ATP binding]; GO:0005634 [Name: nucleus]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>LIM domain kinase 1</t>
+          <t>LIM domain kinase 1-like</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>LIM domain kinase 1 isoform X3</t>
+          <t>LIM domain kinase 1 isoform X2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>N5.HOG0030687</t>
+          <t>N5.HOG0032002</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="D12" t="n">
-        <v>-4.137399677328834</v>
+        <v>1.274928765044614</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.5977397994205895</v>
+        <v>-1.54806206910281</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.9882</v>
+        <v>0.3634</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0118</v>
+        <v>0.6366000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>0.646</v>
+        <v>0.9893999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>0.354</v>
+        <v>0.0106</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>129233408</t>
+          <t>129220871</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>GO:0005737 [Name: cytoplasm]; GO:0005634 [Name: nucleus]; GO:0005524 [Name: ATP binding]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0030036 [Name: actin cytoskeleton organization]; GO:0005515 [Name: protein binding]; GO:0006468 [Name: protein phosphorylation]</t>
+          <t>GO:0005515 [Name: protein binding]; GO:0005829 [Name: cytosol]; GO:0022008 [Name: neurogenesis]</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>LIM domain kinase 1-like</t>
+          <t>BTB/POZ domain-containing protein 6-like</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>LIM domain kinase 1 isoform X2</t>
+          <t>BTB/POZ domain-containing protein 6-A</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>N5.HOG0032002</t>
+          <t>N5.HOG0032852</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D13" t="n">
-        <v>2.315627652613129</v>
+        <v>-3.951967014087926</v>
       </c>
       <c r="E13" t="n">
-        <v>-1.741129233943886</v>
+        <v>0.5403816457665632</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.2209</v>
+        <v>0.9656</v>
       </c>
       <c r="H13" t="n">
-        <v>0.7791</v>
+        <v>0.0344</v>
       </c>
       <c r="I13" t="n">
-        <v>0.9936</v>
+        <v>0.3192</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0064</v>
+        <v>0.6808</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>129226009</t>
+          <t>129218644</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>GO:0005515 [Name: protein binding]; GO:0005829 [Name: cytosol]; GO:0022008 [Name: neurogenesis]; GO:0000932 [Name: P-body]</t>
+          <t>GO:0000407 [Name: pre-autophagosomal structure]; GO:0000045 [Name: autophagosome assembly]; GO:0034497 [Name: protein localization to pre-autophagosomal structure]; GO:0000423 [Name: macromitophagy]; GO:0034727 [Name: piecemeal microautophagy of nucleus]; GO:1990316 [Name: ATG1/ULK1 kinase complex]; GO:0005829 [Name: cytosol]; GO:0019898 [Name: extrinsic component of membrane]</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>BTB/POZ domain-containing protein 3-like</t>
+          <t>autophagy-related protein 13-like</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>BTB/POZ domain-containing protein 6-A</t>
+          <t>autophagy-related protein 13 homolog</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>N5.HOG0032852</t>
+          <t>N5.HOG0034467</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Loss more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="D14" t="n">
-        <v>-4.117592695179181</v>
+        <v>1.667422234094606</v>
       </c>
       <c r="E14" t="n">
-        <v>0.946288800253516</v>
+        <v>-1.28033039179645</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.9872</v>
+        <v>0.0158</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0128</v>
+        <v>0.9842</v>
       </c>
       <c r="I14" t="n">
-        <v>0.2295</v>
+        <v>0.7733</v>
       </c>
       <c r="J14" t="n">
-        <v>0.7705</v>
+        <v>0.2267</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>129218644</t>
+          <t>129230589</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>GO:0000407 [Name: pre-autophagosomal structure]; GO:0000045 [Name: autophagosome assembly]; GO:0034497 [Name: protein localization to pre-autophagosomal structure]; GO:0000423 [Name: macromitophagy]; GO:0034727 [Name: piecemeal microautophagy of nucleus]; GO:1990316 [Name: ATG1/ULK1 kinase complex]; GO:0005829 [Name: cytosol]; GO:0019898 [Name: extrinsic component of membrane]</t>
+          <t>GO:0005875 [Name: microtubule associated complex]; GO:0007409 [Name: axonogenesis]; GO:0045202 [Name: synapse]; GO:0030425 [Name: dendrite]; GO:0003779 [Name: actin binding]; GO:0005829 [Name: cytosol]; GO:0005874 [Name: microtubule]; GO:0000226 [Name: microtubule cytoskeleton organization]; GO:0031114 [Name: regulation of microtubule depolymerization]; GO:0043025 [Name: neuronal cell body]; GO:0016358 [Name: dendrite development]; GO:0008017 [Name: microtubule binding]</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>autophagy-related protein 13-like</t>
+          <t>microtubule-associated protein futsch-like</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>autophagy-related protein 13 homolog</t>
+          <t>microtubule-associated protein futsch</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>N5.HOG0034467</t>
+          <t>N5.HOG0035629</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Loss more likely in orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="D15" t="n">
-        <v>1.689829480176377</v>
+        <v>-1.684498986055916</v>
       </c>
       <c r="E15" t="n">
-        <v>-1.425959551180883</v>
+        <v>1.424655213785957</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1268,42 +1280,42 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.0327</v>
+        <v>0.9002</v>
       </c>
       <c r="H15" t="n">
-        <v>0.9673</v>
+        <v>0.0998</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8366</v>
+        <v>0.0405</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1634</v>
+        <v>0.9595</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>129230589</t>
+          <t>129234338</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>GO:0005875 [Name: microtubule associated complex]; GO:0007409 [Name: axonogenesis]; GO:0045202 [Name: synapse]; GO:0030425 [Name: dendrite]; GO:0003779 [Name: actin binding]; GO:0005829 [Name: cytosol]; GO:0005874 [Name: microtubule]; GO:0000226 [Name: microtubule cytoskeleton organization]; GO:0031114 [Name: regulation of microtubule depolymerization]; GO:0043025 [Name: neuronal cell body]; GO:0016358 [Name: dendrite development]; GO:0008017 [Name: microtubule binding]</t>
+          <t>GO:0000981 [Name: RNA polymerase II transcription factor activity, sequence-specific DNA binding]; GO:0006357 [Name: regulation of transcription from RNA polymerase II promoter]; GO:0000977 [Name: RNA polymerase II regulatory region sequence-specific DNA binding]; GO:0030182 [Name: neuron differentiation]; GO:0005634 [Name: nucleus]</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>microtubule-associated protein futsch-like</t>
+          <t>LIM/homeobox protein Lhx1-like</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>microtubule-associated protein futsch</t>
+          <t>LOW QUALITY PROTEIN: LIM/homeobox protein Lhx1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>N5.HOG0035481</t>
+          <t>N5.HOG0036003</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1312,13 +1324,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D16" t="n">
-        <v>-2.989118479976214</v>
+        <v>-3.79089242176013</v>
       </c>
       <c r="E16" t="n">
-        <v>-1.257140544646757</v>
+        <v>0.5767808481942522</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1326,42 +1338,42 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0.9673</v>
+        <v>0.9523</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0327</v>
+        <v>0.0477</v>
       </c>
       <c r="I16" t="n">
-        <v>0.8546</v>
+        <v>0.4166</v>
       </c>
       <c r="J16" t="n">
-        <v>0.1454</v>
+        <v>0.5834</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>129225528</t>
+          <t>129234391</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>GO:0004550 [Name: nucleoside diphosphate kinase activity]; GO:0006241 [Name: CTP biosynthetic process]; GO:0006183 [Name: GTP biosynthetic process]; GO:0006228 [Name: UTP biosynthetic process]</t>
+          <t>GO:0006164 [Name: purine nucleotide biosynthetic process]; GO:0009156 [Name: ribonucleoside monophosphate biosynthetic process]; GO:0002189 [Name: ribose phosphate diphosphokinase complex]; GO:0005737 [Name: cytoplasm]; GO:0004749 [Name: ribose phosphate diphosphokinase activity]; GO:0006015 [Name: 5-phosphoribose 1-diphosphate biosynthetic process]; GO:0000287 [Name: magnesium ion binding]</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>nucleoside diphosphate kinase-like</t>
+          <t>ribose-phosphate pyrophosphokinase 2-like</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>nucleoside diphosphate kinase</t>
+          <t>ribose-phosphate pyrophosphokinase 2 isoform X2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>N5.HOG0036003</t>
+          <t>N5.HOG0040158</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1370,13 +1382,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D17" t="n">
-        <v>-3.950631580011455</v>
+        <v>-3.126611082576801</v>
       </c>
       <c r="E17" t="n">
-        <v>0.8792919086776682</v>
+        <v>2.889692011031725</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1384,57 +1396,57 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.954</v>
+        <v>0.955</v>
       </c>
       <c r="H17" t="n">
-        <v>0.046</v>
+        <v>0.045</v>
       </c>
       <c r="I17" t="n">
-        <v>0.3946</v>
+        <v>0.1277</v>
       </c>
       <c r="J17" t="n">
-        <v>0.6054</v>
+        <v>0.8723</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>129234391</t>
+          <t>129230758</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>GO:0006164 [Name: purine nucleotide biosynthetic process]; GO:0009156 [Name: ribonucleoside monophosphate biosynthetic process]; GO:0002189 [Name: ribose phosphate diphosphokinase complex]; GO:0005737 [Name: cytoplasm]; GO:0004749 [Name: ribose phosphate diphosphokinase activity]; GO:0006015 [Name: 5-phosphoribose 1-diphosphate biosynthetic process]; GO:0000287 [Name: magnesium ion binding]</t>
+          <t>GO:0006897 [Name: endocytosis]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005886 [Name: plasma membrane]; GO:0090263 [Name: positive regulation of canonical Wnt signaling pathway]; GO:0005524 [Name: ATP binding]; GO:0005634 [Name: nucleus]; GO:0007165 [Name: signal transduction]; GO:0005737 [Name: cytoplasm]; GO:0018105 [Name: peptidyl-serine phosphorylation]</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>ribose-phosphate pyrophosphokinase 2-like</t>
+          <t>casein kinase I gish</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>ribose-phosphate pyrophosphokinase 2 isoform X2</t>
+          <t>casein kinase I isoform X4</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>N5.HOG0036231</t>
+          <t>N5.HOG0046893</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Loss more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="D18" t="n">
-        <v>-1.553406126533798</v>
+        <v>1.420299028263379</v>
       </c>
       <c r="E18" t="n">
-        <v>1.283511440663914</v>
+        <v>-0.8015196595948118</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1442,100 +1454,100 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.9765</v>
+        <v>0.0443</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0235</v>
+        <v>0.9557</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2225</v>
+        <v>0.7981</v>
       </c>
       <c r="J18" t="n">
-        <v>0.7775</v>
+        <v>0.2019</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>129220274</t>
+          <t>129224651</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>GO:0051966 [Name: regulation of synaptic transmission, glutamatergic]; GO:0007216 [Name: G-protein coupled glutamate receptor signaling pathway]; GO:0016020 [Name: membrane]; GO:0001641 [Name: group II metabotropic glutamate receptor activity]</t>
+          <t>GO:0008613 [Name: diuretic hormone activity]; GO:0001664 [Name: G-protein coupled receptor binding]; GO:0007589 [Name: body fluid secretion]; GO:0005615 [Name: extracellular space]</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>metabotropic glutamate receptor 2-like</t>
+          <t>diuretic hormone class 2-like</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>metabotropic glutamate receptor 3 isoform X1</t>
+          <t>diuretic hormone class 2-like</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>N5.HOG0038912</t>
+          <t>N5.HOG0048186</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Duplication more likely in orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D19" t="n">
-        <v>1.793712319835324</v>
+        <v>-1.867837837277505</v>
       </c>
       <c r="E19" t="n">
-        <v>1.523147351558712</v>
+        <v>-2.544953891852447</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0.1052</v>
+        <v>0.7672</v>
       </c>
       <c r="H19" t="n">
-        <v>0.8948</v>
+        <v>0.2328</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0466</v>
+        <v>0.9968</v>
       </c>
       <c r="J19" t="n">
-        <v>0.9534</v>
+        <v>0.0032</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>129227546</t>
+          <t>129218892</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>GO:0005509 [Name: calcium ion binding]</t>
+          <t>GO:0001678 [Name: cellular glucose homeostasis]; GO:0005739 [Name: mitochondrion]; GO:0006096 [Name: glycolytic process]; GO:0051156 [Name: glucose 6-phosphate metabolic process]; GO:0019158 [Name: mannokinase activity]; GO:0005829 [Name: cytosol]; GO:0008865 [Name: fructokinase activity]; GO:0004340 [Name: glucokinase activity]; GO:0005524 [Name: ATP binding]; GO:0005536 [Name: glucose binding]</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>neurogenic locus notch homolog protein 1-like</t>
+          <t>hexokinase-1-like</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>adhesive plaque matrix protein 2</t>
+          <t>hexokinase type 2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>N5.HOG0040158</t>
+          <t>N5.HOG0048441</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1544,129 +1556,129 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="D20" t="n">
-        <v>-3.304074752495731</v>
+        <v>-1.701769774016</v>
       </c>
       <c r="E20" t="n">
-        <v>3.1802244726272</v>
+        <v>-0.2690227423510625</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.9577</v>
+        <v>0.9536</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0423</v>
+        <v>0.0464</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1199</v>
+        <v>0.6342</v>
       </c>
       <c r="J20" t="n">
-        <v>0.8801</v>
+        <v>0.3658</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>129230758</t>
+          <t>129219213</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>GO:0006897 [Name: endocytosis]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005886 [Name: plasma membrane]; GO:0090263 [Name: positive regulation of canonical Wnt signaling pathway]; GO:0005524 [Name: ATP binding]; GO:0005634 [Name: nucleus]; GO:0007165 [Name: signal transduction]; GO:0005737 [Name: cytoplasm]; GO:0018105 [Name: peptidyl-serine phosphorylation]</t>
+          <t>GO:0098802 [Name: plasma membrane receptor complex]; GO:0046330 [Name: positive regulation of JNK cascade]; GO:0061630 [Name: ubiquitin protein ligase activity]; GO:0043122 [Name: regulation of I-kappaB kinase/NF-kappaB signaling]; GO:0033209 [Name: tumor necrosis factor-mediated signaling pathway]; GO:0070534 [Name: protein K63-linked ubiquitination]</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>casein kinase I gish</t>
+          <t>E3 ubiquitin-protein ligase NRDP1 elgi</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>casein kinase I isoform X4</t>
+          <t>E3 ubiquitin-protein ligase NRDP1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>N5.HOG0041634</t>
+          <t>N5.HOG0048897</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Loss more likely in orb-weavers, duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="D21" t="n">
-        <v>-3.991082659384722</v>
+        <v>1.528545174493033</v>
       </c>
       <c r="E21" t="n">
-        <v>2.159486406107594</v>
+        <v>-2.106825375295115</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0.9694</v>
+        <v>0.0361</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0305</v>
+        <v>0.9639</v>
       </c>
       <c r="I21" t="n">
-        <v>0.08</v>
+        <v>0.9913</v>
       </c>
       <c r="J21" t="n">
-        <v>0.92</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>129227265</t>
+          <t>129217740</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>GO:0016311 [Name: dephosphorylation]; GO:0052629 [Name: phosphatidylinositol-3,5-bisphosphate 3-phosphatase activity]; GO:0010506 [Name: regulation of autophagy]; GO:0019903 [Name: protein phosphatase binding]</t>
+          <t>GO:0008277 [Name: regulation of G-protein coupled receptor protein signaling pathway]; GO:0035556 [Name: intracellular signal transduction]; GO:0007186 [Name: G-protein coupled receptor signaling pathway]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>myotubularin-related protein 3-like</t>
+          <t>regulator of G-protein signaling 7-like</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>phosphatidylinositol-3,5-bisphosphate 3-phosphatase MTMR3</t>
+          <t>regulator of G-protein signaling 7 isoform X2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>N5.HOG0045525</t>
+          <t>N5.HOG0050702</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="D22" t="n">
-        <v>-1.268925667853019</v>
+        <v>0.8668912516335915</v>
       </c>
       <c r="E22" t="n">
-        <v>1.526783060512084</v>
+        <v>-1.480245404596741</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1674,57 +1686,57 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0.9646</v>
+        <v>0.2156</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0354</v>
+        <v>0.7843</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1123</v>
+        <v>0.9888</v>
       </c>
       <c r="J22" t="n">
-        <v>0.8877</v>
+        <v>0.0112</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>129230436</t>
+          <t>129224238</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>GO:0005829 [Name: cytosol]; GO:0004694 [Name: eukaryotic translation initiation factor 2alpha kinase activity]; GO:0000077 [Name: DNA damage checkpoint]; GO:0010998 [Name: regulation of translational initiation by eIF2 alpha phosphorylation]; GO:0005524 [Name: ATP binding]; GO:0005515 [Name: protein binding]</t>
+          <t>GO:0043491 [Name: protein kinase B signaling]; GO:0005942 [Name: phosphatidylinositol 3-kinase complex]; GO:0035005 [Name: 1-phosphatidylinositol-4-phosphate 3-kinase activity]; GO:0005886 [Name: plasma membrane]; GO:0048015 [Name: phosphatidylinositol-mediated signaling]; GO:0005737 [Name: cytoplasm]; GO:0016303 [Name: 1-phosphatidylinositol-3-kinase activity]; GO:0016477 [Name: cell migration]; GO:0036092 [Name: phosphatidylinositol-3-phosphate biosynthetic process]</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>eukaryotic translation initiation factor 2 alpha kinase Gcn2</t>
+          <t>phosphatidylinositol 3-kinase 92E</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>eIF-2-alpha kinase GCN2</t>
+          <t>phosphatidylinositol 4,5-bisphosphate 3-kinase catalytic subunit delta isoform</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>N5.HOG0046893</t>
+          <t>N5.HOG0051572</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Loss more likely in orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D23" t="n">
-        <v>1.745709484732493</v>
+        <v>-2.647951965886426</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.9296068173722239</v>
+        <v>1.636211633780647</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1732,100 +1744,100 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>0.0262</v>
+        <v>0.9328</v>
       </c>
       <c r="H23" t="n">
-        <v>0.9738</v>
+        <v>0.0672</v>
       </c>
       <c r="I23" t="n">
-        <v>0.8011</v>
+        <v>0.0365</v>
       </c>
       <c r="J23" t="n">
-        <v>0.1989</v>
+        <v>0.9635</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>129224651</t>
+          <t>129228238</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>GO:0008613 [Name: diuretic hormone activity]; GO:0001664 [Name: G-protein coupled receptor binding]; GO:0007589 [Name: body fluid secretion]; GO:0005615 [Name: extracellular space]</t>
+          <t>GO:0001726 [Name: ruffle]; GO:0004439 [Name: phosphatidylinositol-4,5-bisphosphate 5-phosphatase activity]; GO:0005737 [Name: cytoplasm]; GO:0046856 [Name: phosphatidylinositol dephosphorylation]; GO:0005886 [Name: plasma membrane]</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>diuretic hormone class 2-like</t>
+          <t>inositol polyphosphate 5-phosphatase K-like</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>diuretic hormone class 2-like</t>
+          <t>phosphatidylinositol 4,5-bisphosphate 5-phosphatase A isoform X4</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>N5.HOG0048186</t>
+          <t>N5.HOG0053555</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers, duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>-2.010017487192618</v>
+        <v>-3.03255284649051</v>
       </c>
       <c r="E24" t="n">
-        <v>-2.677562794397825</v>
+        <v>-1.696958693304238</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes for loss; no for duplication</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>0.801</v>
+        <v>0.9943</v>
       </c>
       <c r="H24" t="n">
-        <v>0.199</v>
+        <v>0.0057</v>
       </c>
       <c r="I24" t="n">
-        <v>0.9985000000000001</v>
+        <v>0.9959</v>
       </c>
       <c r="J24" t="n">
-        <v>0.0015</v>
+        <v>0.0041</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>129218892</t>
+          <t>129228121</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>GO:0001678 [Name: cellular glucose homeostasis]; GO:0005739 [Name: mitochondrion]; GO:0006096 [Name: glycolytic process]; GO:0051156 [Name: glucose 6-phosphate metabolic process]; GO:0019158 [Name: mannokinase activity]; GO:0005829 [Name: cytosol]; GO:0008865 [Name: fructokinase activity]; GO:0004340 [Name: glucokinase activity]; GO:0005524 [Name: ATP binding]; GO:0005536 [Name: glucose binding]</t>
+          <t>GO:0004749 [Name: ribose phosphate diphosphokinase activity]; GO:0006015 [Name: 5-phosphoribose 1-diphosphate biosynthetic process]; GO:0005737 [Name: cytoplasm]; GO:0006164 [Name: purine nucleotide biosynthetic process]; GO:0000287 [Name: magnesium ion binding]; GO:0002189 [Name: ribose phosphate diphosphokinase complex]</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>hexokinase-1-like</t>
+          <t>phosphoribosyl pyrophosphate synthase-associated protein 2-like</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>hexokinase type 2</t>
+          <t>phosphoribosyl pyrophosphate synthase-associated protein 2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>N5.HOG0050702</t>
+          <t>N5.HOG0054227</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1834,13 +1846,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D25" t="n">
-        <v>0.7351914124605211</v>
+        <v>0.3349693480177507</v>
       </c>
       <c r="E25" t="n">
-        <v>-1.648705150156974</v>
+        <v>-1.425149241466285</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1848,57 +1860,57 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0.3011</v>
+        <v>0.2231</v>
       </c>
       <c r="H25" t="n">
-        <v>0.6989</v>
+        <v>0.7768</v>
       </c>
       <c r="I25" t="n">
-        <v>0.9931</v>
+        <v>0.9701</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0069</v>
+        <v>0.0299</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>129224238</t>
+          <t>129224230</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>GO:0043491 [Name: protein kinase B signaling]; GO:0005942 [Name: phosphatidylinositol 3-kinase complex]; GO:0035005 [Name: 1-phosphatidylinositol-4-phosphate 3-kinase activity]; GO:0005886 [Name: plasma membrane]; GO:0048015 [Name: phosphatidylinositol-mediated signaling]; GO:0005737 [Name: cytoplasm]; GO:0016303 [Name: 1-phosphatidylinositol-3-kinase activity]; GO:0016477 [Name: cell migration]; GO:0036092 [Name: phosphatidylinositol-3-phosphate biosynthetic process]</t>
+          <t>GO:0035091 [Name: phosphatidylinositol binding]; GO:0008270 [Name: zinc ion binding]; GO:0003676 [Name: nucleic acid binding]</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>phosphatidylinositol 3-kinase 92E</t>
+          <t>zinc finger CCHC domain-containing protein 2-like</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>phosphatidylinositol 4,5-bisphosphate 3-kinase catalytic subunit delta isoform</t>
+          <t>zinc finger CCHC domain-containing protein 2 isoform X2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>N5.HOG0051572</t>
+          <t>N5.HOG0054901</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Duplication more likely in orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>69</v>
+        <v>96</v>
       </c>
       <c r="D26" t="n">
-        <v>-2.829040507600939</v>
+        <v>-1.25678417448257</v>
       </c>
       <c r="E26" t="n">
-        <v>1.978409021475309</v>
+        <v>-2.075131227901787</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1906,448 +1918,448 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0.9157999999999999</v>
+        <v>0.7378</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0842</v>
+        <v>0.2621</v>
       </c>
       <c r="I26" t="n">
-        <v>0.0203</v>
+        <v>0.9696</v>
       </c>
       <c r="J26" t="n">
-        <v>0.9797</v>
+        <v>0.0304</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>129228238</t>
+          <t>129227017</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>GO:0001726 [Name: ruffle]; GO:0004439 [Name: phosphatidylinositol-4,5-bisphosphate 5-phosphatase activity]; GO:0005737 [Name: cytoplasm]; GO:0046856 [Name: phosphatidylinositol dephosphorylation]; GO:0005886 [Name: plasma membrane]</t>
+          <t>GO:0007165 [Name: signal transduction]; GO:0005737 [Name: cytoplasm]; GO:0005634 [Name: nucleus]; GO:0018105 [Name: peptidyl-serine phosphorylation]; GO:0006897 [Name: endocytosis]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005524 [Name: ATP binding]</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>inositol polyphosphate 5-phosphatase K-like</t>
+          <t>casein kinase I-like</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>phosphatidylinositol 4,5-bisphosphate 5-phosphatase A isoform X4</t>
+          <t>casein kinase I</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>N5.HOG0052976</t>
+          <t>N5.HOG0058078</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D27" t="n">
-        <v>-3.990831611641441</v>
+        <v>-0.7256542955276075</v>
       </c>
       <c r="E27" t="n">
-        <v>1.115541354696966</v>
+        <v>1.811869176606395</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>0.9752</v>
+        <v>0.5648</v>
       </c>
       <c r="H27" t="n">
-        <v>0.0248</v>
+        <v>0.4352</v>
       </c>
       <c r="I27" t="n">
-        <v>0.3678</v>
+        <v>0.0498</v>
       </c>
       <c r="J27" t="n">
-        <v>0.6322</v>
+        <v>0.9502</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>129219959</t>
+          <t>129225594</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>GO:0006914 [Name: autophagy]; GO:0034271 [Name: phosphatidylinositol 3-kinase complex, class III, type I]; GO:0045324 [Name: late endosome to vacuole transport]; GO:0000045 [Name: autophagosome assembly]; GO:0000407 [Name: pre-autophagosomal structure]; GO:0006995 [Name: cellular response to nitrogen starvation]; GO:0034272 [Name: phosphatidylinositol 3-kinase complex, class III, type II]</t>
+          <t>GO:0030425 [Name: dendrite]; GO:0048168 [Name: regulation of neuronal synaptic plasticity]; GO:0031175 [Name: neuron projection development]</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>beclin-1-like</t>
+          <t>neurochondrin homolog</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>beclin-1</t>
+          <t>neurochondrin homolog</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>N5.HOG0053555</t>
+          <t>N5.HOG0058262</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers, duplication more likely in non-orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D28" t="n">
-        <v>-3.174598677231178</v>
+        <v>-3.486151905508599</v>
       </c>
       <c r="E28" t="n">
-        <v>-1.212892934558675</v>
+        <v>1.530248754206848</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Yes for loss; no for duplication</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0.9983</v>
+        <v>0.8943</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0017</v>
+        <v>0.1057</v>
       </c>
       <c r="I28" t="n">
-        <v>0.9615</v>
+        <v>0.0228</v>
       </c>
       <c r="J28" t="n">
-        <v>0.0385</v>
+        <v>0.9772</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>129228121</t>
+          <t>129215997</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>GO:0004749 [Name: ribose phosphate diphosphokinase activity]; GO:0006015 [Name: 5-phosphoribose 1-diphosphate biosynthetic process]; GO:0005737 [Name: cytoplasm]; GO:0006164 [Name: purine nucleotide biosynthetic process]; GO:0000287 [Name: magnesium ion binding]; GO:0002189 [Name: ribose phosphate diphosphokinase complex]</t>
+          <t>GO:0006470 [Name: protein dephosphorylation]; GO:0043169 [Name: cation binding]; GO:0004722 [Name: protein serine/threonine phosphatase activity]</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>phosphoribosyl pyrophosphate synthase-associated protein 2-like</t>
+          <t>TGF-beta-activated kinase 1 and MAP3K7-binding protein 1-like</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>phosphoribosyl pyrophosphate synthase-associated protein 2</t>
+          <t>TGF-beta-activated kinase 1 and MAP3K7-binding protein 1 isoform X1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>N5.HOG0054227</t>
+          <t>N5.HOG0059968</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>98</v>
+        <v>75</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2077358748847513</v>
+        <v>-3.96907534691269</v>
       </c>
       <c r="E29" t="n">
-        <v>-1.610648918764712</v>
+        <v>0.1487060270050904</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>0.4018</v>
+        <v>0.9863</v>
       </c>
       <c r="H29" t="n">
-        <v>0.5981</v>
+        <v>0.0137</v>
       </c>
       <c r="I29" t="n">
-        <v>0.983</v>
+        <v>0.3737</v>
       </c>
       <c r="J29" t="n">
-        <v>0.017</v>
+        <v>0.6263</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>129224230</t>
+          <t>129224556</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>GO:0035091 [Name: phosphatidylinositol binding]; GO:0008270 [Name: zinc ion binding]; GO:0003676 [Name: nucleic acid binding]</t>
+          <t>GO:0005886 [Name: plasma membrane]; GO:0046854 [Name: phosphatidylinositol phosphorylation]; GO:0072659 [Name: protein localization to plasma membrane]</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>zinc finger CCHC domain-containing protein 2-like</t>
+          <t>PI4KA lipid kinase complex subunit hyccin</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>zinc finger CCHC domain-containing protein 2 isoform X2</t>
+          <t>hyccin</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>N5.HOG0054901</t>
+          <t>N5.HOG0060288</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="D30" t="n">
-        <v>-1.386073711129391</v>
+        <v>-2.702517333918679</v>
       </c>
       <c r="E30" t="n">
-        <v>-2.230258112126691</v>
+        <v>-0.487062078600888</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0.8475</v>
+        <v>0.9528</v>
       </c>
       <c r="H30" t="n">
-        <v>0.1525</v>
+        <v>0.0472</v>
       </c>
       <c r="I30" t="n">
-        <v>0.9617</v>
+        <v>0.5478</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0382</v>
+        <v>0.4522</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>129227017</t>
+          <t>129222137</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>GO:0007165 [Name: signal transduction]; GO:0005737 [Name: cytoplasm]; GO:0005634 [Name: nucleus]; GO:0018105 [Name: peptidyl-serine phosphorylation]; GO:0006897 [Name: endocytosis]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005524 [Name: ATP binding]</t>
+          <t>GO:0005634 [Name: nucleus]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0044773 [Name: mitotic DNA damage checkpoint]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>casein kinase I-like</t>
+          <t>cell division cycle 7-related protein kinase-like</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>casein kinase I</t>
+          <t>cell division cycle 7-related protein kinase isoform X1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>N5.HOG0055160</t>
+          <t>N5.HOG0061119</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="D31" t="n">
-        <v>-3.176356469322564</v>
+        <v>1.071261968122538</v>
       </c>
       <c r="E31" t="n">
-        <v>0.0348238335131094</v>
+        <v>-2.054862693041546</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>0.9607</v>
+        <v>0.1148</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0393</v>
+        <v>0.8852</v>
       </c>
       <c r="I31" t="n">
-        <v>0.583</v>
+        <v>0.9719</v>
       </c>
       <c r="J31" t="n">
-        <v>0.4168</v>
+        <v>0.0281</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>129216986</t>
+          <t>129225556</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>GO:0005524 [Name: ATP binding]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0006468 [Name: protein phosphorylation]</t>
+          <t>GO:0006811 [Name: ion transport]; GO:0043005 [Name: neuron projection]; GO:0035235 [Name: ionotropic glutamate receptor signaling pathway]; GO:0042391 [Name: regulation of membrane potential]; GO:0005886 [Name: plasma membrane]; GO:0017146 [Name: NMDA selective glutamate receptor complex]; GO:0045202 [Name: synapse]; GO:0004972 [Name: NMDA glutamate receptor activity]; GO:0007268 [Name: chemical synaptic transmission]</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>cAMP-dependent protein kinase catalytic subunit 3-like</t>
+          <t>glutamate [NMDA] receptor subunit 1-like</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>cAMP-dependent protein kinase catalytic subunit 3 isoform X1</t>
+          <t>glutamate [NMDA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>N5.HOG0059968</t>
+          <t>N5.HOG0061199</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="D32" t="n">
-        <v>-4.135386034876563</v>
+        <v>-0.7254076171249628</v>
       </c>
       <c r="E32" t="n">
-        <v>0.0140837004800931</v>
+        <v>-2.022475220611714</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>0.9966</v>
+        <v>0.5127</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0034</v>
+        <v>0.4873</v>
       </c>
       <c r="I32" t="n">
-        <v>0.463</v>
+        <v>0.9658</v>
       </c>
       <c r="J32" t="n">
-        <v>0.537</v>
+        <v>0.0342</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>129224556</t>
+          <t>129227869</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>GO:0005886 [Name: plasma membrane]; GO:0046854 [Name: phosphatidylinositol phosphorylation]; GO:0072659 [Name: protein localization to plasma membrane]</t>
+          <t>GO:0046579 [Name: positive regulation of Ras protein signal transduction]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0006468 [Name: protein phosphorylation]</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>PI4KA lipid kinase complex subunit hyccin</t>
+          <t>serine/threonine-protein kinase 19-like</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>hyccin</t>
+          <t>inactive serine/threonine-protein kinase 19</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>N5.HOG0060288</t>
+          <t>N5.HOG0062578</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="D33" t="n">
-        <v>-2.88730016443721</v>
+        <v>0.3349693480177507</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.6140855930845586</v>
+        <v>-2.369802435297485</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>0.9636</v>
+        <v>0.2231</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0364</v>
+        <v>0.7768</v>
       </c>
       <c r="I33" t="n">
-        <v>0.5561</v>
+        <v>0.9826</v>
       </c>
       <c r="J33" t="n">
-        <v>0.4439</v>
+        <v>0.0174</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>129222137</t>
+          <t>129216091</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>GO:0005634 [Name: nucleus]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0044773 [Name: mitotic DNA damage checkpoint]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]</t>
+          <t>GO:0019543 [Name: propionate catabolic process]; GO:0005829 [Name: cytosol]; GO:0004613 [Name: phosphoenolpyruvate carboxykinase (GTP) activity]; GO:0005525 [Name: GTP binding]; GO:0046327 [Name: glycerol biosynthetic process from pyruvate]; GO:0006094 [Name: gluconeogenesis]; GO:0030145 [Name: manganese ion binding]; GO:0032869 [Name: cellular response to insulin stimulus]; GO:0042594 [Name: response to starvation]; GO:0070365 [Name: hepatocyte differentiation]; GO:0071333 [Name: cellular response to glucose stimulus]; GO:0071549 [Name: cellular response to dexamethasone stimulus]</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>cell division cycle 7-related protein kinase-like</t>
+          <t>phosphoenolpyruvate carboxykinase, cytosolic [GTP]-like</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>cell division cycle 7-related protein kinase isoform X1</t>
+          <t>phosphoenolpyruvate carboxykinase, cytosolic [GTP</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>N5.HOG0061119</t>
+          <t>N5.HOG0063077</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2356,114 +2368,114 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="D34" t="n">
-        <v>1.15566410053318</v>
+        <v>-1.260837948086103</v>
       </c>
       <c r="E34" t="n">
-        <v>-2.195040279343629</v>
+        <v>-1.784817696803436</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>0.1291</v>
+        <v>0.7608</v>
       </c>
       <c r="H34" t="n">
-        <v>0.8709</v>
+        <v>0.2392</v>
       </c>
       <c r="I34" t="n">
-        <v>0.9678</v>
+        <v>0.9733000000000001</v>
       </c>
       <c r="J34" t="n">
-        <v>0.0322</v>
+        <v>0.0267</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>129225556</t>
+          <t>129219268</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>GO:0006811 [Name: ion transport]; GO:0043005 [Name: neuron projection]; GO:0035235 [Name: ionotropic glutamate receptor signaling pathway]; GO:0042391 [Name: regulation of membrane potential]; GO:0005886 [Name: plasma membrane]; GO:0017146 [Name: NMDA selective glutamate receptor complex]; GO:0045202 [Name: synapse]; GO:0004972 [Name: NMDA glutamate receptor activity]; GO:0007268 [Name: chemical synaptic transmission]</t>
+          <t>GO:0043025 [Name: neuronal cell body]; GO:0045727 [Name: positive regulation of translation]; GO:0043197 [Name: dendritic spine]; GO:0048814 [Name: regulation of dendrite morphogenesis]; GO:0016020 [Name: membrane]; GO:0071598 [Name: neuronal ribonucleoprotein granule]; GO:0003730 [Name: mRNA 3'-UTR binding]; GO:0030424 [Name: axon]; GO:0042803 [Name: protein homodimerization activity]; GO:0043488 [Name: regulation of mRNA stability]; GO:0060998 [Name: regulation of dendritic spine development]; GO:0099578 [Name: regulation of translation at postsynapse, modulating synaptic transmission]; GO:0008089 [Name: anterograde axonal transport]; GO:0014069 [Name: postsynaptic density]; GO:0045182 [Name: translation regulator activity]; GO:0005634 [Name: nucleus]; GO:0007417 [Name: central nervous system development]; GO:0017148 [Name: negative regulation of translation]; GO:1905244 [Name: regulation of modification of synaptic structure]</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>glutamate [NMDA] receptor subunit 1-like</t>
+          <t>fragile X messenger ribonucleoprotein 1 homolog</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>glutamate [NMDA</t>
+          <t>RNA-binding protein FXR1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>N5.HOG0061199</t>
+          <t>N5.HOG0066939</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.8536324806155225</v>
+        <v>-2.650703581186066</v>
       </c>
       <c r="E35" t="n">
-        <v>-2.175810617809173</v>
+        <v>0.939259027269308</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>0.6731</v>
+        <v>0.9714</v>
       </c>
       <c r="H35" t="n">
-        <v>0.3268</v>
+        <v>0.0286</v>
       </c>
       <c r="I35" t="n">
-        <v>0.9797</v>
+        <v>0.0699</v>
       </c>
       <c r="J35" t="n">
-        <v>0.0203</v>
+        <v>0.9301</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>129227869</t>
+          <t>129228009</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>GO:0046579 [Name: positive regulation of Ras protein signal transduction]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0006468 [Name: protein phosphorylation]</t>
+          <t>GO:0015250 [Name: water channel activity]; GO:0055085 [Name: transmembrane transport]; GO:0005886 [Name: plasma membrane]</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>serine/threonine-protein kinase 19-like</t>
+          <t>neurogenic protein big brain-like</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>inactive serine/threonine-protein kinase 19</t>
+          <t>aquaporin AQPAe.a</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>N5.HOG0062578</t>
+          <t>N5.HOG0067099</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2472,13 +2484,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="D36" t="n">
-        <v>0.2077358748847513</v>
+        <v>2.257461790658672</v>
       </c>
       <c r="E36" t="n">
-        <v>-2.516941519898598</v>
+        <v>-2.780945563596604</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2486,57 +2498,57 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>0.4018</v>
+        <v>0.083</v>
       </c>
       <c r="H36" t="n">
-        <v>0.5981</v>
+        <v>0.917</v>
       </c>
       <c r="I36" t="n">
-        <v>0.9723000000000001</v>
+        <v>0.9689</v>
       </c>
       <c r="J36" t="n">
-        <v>0.0276</v>
+        <v>0.0311</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>129216091</t>
+          <t>129225034</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>GO:0019543 [Name: propionate catabolic process]; GO:0005829 [Name: cytosol]; GO:0004613 [Name: phosphoenolpyruvate carboxykinase (GTP) activity]; GO:0005525 [Name: GTP binding]; GO:0046327 [Name: glycerol biosynthetic process from pyruvate]; GO:0006094 [Name: gluconeogenesis]; GO:0030145 [Name: manganese ion binding]; GO:0032869 [Name: cellular response to insulin stimulus]; GO:0042594 [Name: response to starvation]; GO:0070365 [Name: hepatocyte differentiation]; GO:0071333 [Name: cellular response to glucose stimulus]; GO:0071549 [Name: cellular response to dexamethasone stimulus]</t>
+          <t>GO:0005737 [Name: cytoplasm]; GO:0019901 [Name: protein kinase binding]; GO:0045737 [Name: positive regulation of cyclin-dependent protein serine/threonine kinase activity]; GO:0061575 [Name: cyclin-dependent protein serine/threonine kinase activator activity]; GO:0032147 [Name: activation of protein kinase activity]; GO:0016533 [Name: cyclin-dependent protein kinase 5 holoenzyme complex]</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>phosphoenolpyruvate carboxykinase, cytosolic [GTP]-like</t>
+          <t>Cdk5 activator-like protein</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>phosphoenolpyruvate carboxykinase, cytosolic [GTP</t>
+          <t>cyclin-dependent kinase 5 activator 1 isoform X1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>N5.HOG0063077</t>
+          <t>N5.HOG0068715</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="D37" t="n">
-        <v>-1.390137982015466</v>
+        <v>-2.162736198321358</v>
       </c>
       <c r="E37" t="n">
-        <v>-1.921689414675522</v>
+        <v>0.7122931788181197</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2544,603 +2556,93 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>0.8818</v>
+        <v>0.991</v>
       </c>
       <c r="H37" t="n">
-        <v>0.1182</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="I37" t="n">
-        <v>0.9594</v>
+        <v>0.2442</v>
       </c>
       <c r="J37" t="n">
-        <v>0.0404</v>
+        <v>0.7558</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>129219268</t>
+          <t>129232140</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>GO:0043025 [Name: neuronal cell body]; GO:0045727 [Name: positive regulation of translation]; GO:0043197 [Name: dendritic spine]; GO:0048814 [Name: regulation of dendrite morphogenesis]; GO:0016020 [Name: membrane]; GO:0071598 [Name: neuronal ribonucleoprotein granule]; GO:0003730 [Name: mRNA 3'-UTR binding]; GO:0030424 [Name: axon]; GO:0042803 [Name: protein homodimerization activity]; GO:0043488 [Name: regulation of mRNA stability]; GO:0060998 [Name: regulation of dendritic spine development]; GO:0099578 [Name: regulation of translation at postsynapse, modulating synaptic transmission]; GO:0008089 [Name: anterograde axonal transport]; GO:0014069 [Name: postsynaptic density]; GO:0045182 [Name: translation regulator activity]; GO:0005634 [Name: nucleus]; GO:0007417 [Name: central nervous system development]; GO:0017148 [Name: negative regulation of translation]; GO:1905244 [Name: regulation of modification of synaptic structure]</t>
+          <t>GO:0004930 [Name: G-protein coupled receptor activity]; GO:0007186 [Name: G-protein coupled receptor signaling pathway]; GO:0016020 [Name: membrane]</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>fragile X messenger ribonucleoprotein 1 homolog</t>
+          <t>probable G-protein coupled receptor AH9.1</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>RNA-binding protein FXR1</t>
+          <t>probable G-protein coupled receptor AH9.1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>N5.HOG0064389</t>
+          <t>N5.HOG0068937</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Loss more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D38" t="n">
-        <v>-3.177654618970608</v>
+        <v>1.716305137494582</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.192194723936545</v>
+        <v>-0.2263921591536401</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>0.9562</v>
+        <v>0.0063</v>
       </c>
       <c r="H38" t="n">
-        <v>0.0438</v>
+        <v>0.9937</v>
       </c>
       <c r="I38" t="n">
-        <v>0.617</v>
+        <v>0.5667</v>
       </c>
       <c r="J38" t="n">
-        <v>0.383</v>
+        <v>0.4333</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>129233173</t>
+          <t>129225023</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>GO:0008254 [Name: 3'-nucleotidase activity]; GO:0046854 [Name: phosphatidylinositol phosphorylation]; GO:0012505 [Name: endomembrane system]</t>
+          <t>GO:0007218 [Name: neuropeptide signaling pathway]</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>inositol monophosphatase 3-like</t>
+          <t>FMRFamide propeptide</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>inositol monophosphatase 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>N5.HOG0065326</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Loss more likely in non-orb-weavers</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>77</v>
-      </c>
-      <c r="D39" t="n">
-        <v>-3.992560789633913</v>
-      </c>
-      <c r="E39" t="n">
-        <v>0.6409238946601564</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>0.9708</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0.0291</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0.2429</v>
-      </c>
-      <c r="J39" t="n">
-        <v>0.7571</v>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>129234570</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>GO:0045199 [Name: maintenance of epithelial cell apical/basal polarity]; GO:0007269 [Name: neurotransmitter secretion]; GO:0005515 [Name: protein binding]; GO:0016323 [Name: basolateral plasma membrane]; GO:1903361 [Name: protein localization to basolateral plasma membrane]; GO:0005911 [Name: cell-cell junction]; GO:0045202 [Name: synapse]</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>L27 and PDZ_signaling domain-containing protein veli</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>protein lin-7 homolog C</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>N5.HOG0066668</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Duplication more likely in orb-weavers</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>95</v>
-      </c>
-      <c r="D40" t="n">
-        <v>-0.2776346042345049</v>
-      </c>
-      <c r="E40" t="n">
-        <v>2.132695234890605</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0.4375</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0.0287</v>
-      </c>
-      <c r="J40" t="n">
-        <v>0.9713000000000001</v>
-      </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>uncharacterized protein</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>N5.HOG0066939</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Loss more likely in non-orb-weavers</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>69</v>
-      </c>
-      <c r="D41" t="n">
-        <v>-2.832035136767834</v>
-      </c>
-      <c r="E41" t="n">
-        <v>1.207945256606876</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>0.9755</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0.0245</v>
-      </c>
-      <c r="I41" t="n">
-        <v>0.0512</v>
-      </c>
-      <c r="J41" t="n">
-        <v>0.9488</v>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>129228009</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>GO:0015250 [Name: water channel activity]; GO:0055085 [Name: transmembrane transport]; GO:0005886 [Name: plasma membrane]</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>neurogenic protein big brain-like</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>aquaporin AQPAe.a</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>N5.HOG0067099</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Duplication more likely in non-orb-weavers</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>56</v>
-      </c>
-      <c r="D42" t="n">
-        <v>2.637280863253797</v>
-      </c>
-      <c r="E42" t="n">
-        <v>-2.916447723490454</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>0.0624</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0.9376</v>
-      </c>
-      <c r="I42" t="n">
-        <v>0.9540999999999999</v>
-      </c>
-      <c r="J42" t="n">
-        <v>0.0458</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>129225034</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>GO:0005737 [Name: cytoplasm]; GO:0019901 [Name: protein kinase binding]; GO:0045737 [Name: positive regulation of cyclin-dependent protein serine/threonine kinase activity]; GO:0061575 [Name: cyclin-dependent protein serine/threonine kinase activator activity]; GO:0032147 [Name: activation of protein kinase activity]; GO:0016533 [Name: cyclin-dependent protein kinase 5 holoenzyme complex]</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>Cdk5 activator-like protein</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>cyclin-dependent kinase 5 activator 1 isoform X1</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>N5.HOG0068366</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Loss more likely in non-orb-weavers</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>79</v>
-      </c>
-      <c r="D43" t="n">
-        <v>-2.661432670165445</v>
-      </c>
-      <c r="E43" t="n">
-        <v>0.5412845769453301</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>0.9598</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0.0402</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0.2621</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0.7379</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>129218629</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>GO:0007169 [Name: transmembrane receptor protein tyrosine kinase signaling pathway]; GO:0043410 [Name: positive regulation of MAPK cascade]; GO:0005737 [Name: cytoplasm]</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>docking protein 3-like</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>docking protein 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>N5.HOG0068715</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Loss more likely in non-orb-weavers</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>83</v>
-      </c>
-      <c r="D44" t="n">
-        <v>-2.309868234313403</v>
-      </c>
-      <c r="E44" t="n">
-        <v>0.9319025225028508</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>0.9958</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0.0042</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0.1128</v>
-      </c>
-      <c r="J44" t="n">
-        <v>0.8872</v>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>129232140</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>GO:0004930 [Name: G-protein coupled receptor activity]; GO:0007186 [Name: G-protein coupled receptor signaling pathway]; GO:0016020 [Name: membrane]</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>probable G-protein coupled receptor AH9.1</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>probable G-protein coupled receptor AH9.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>N5.HOG0068937</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Loss more likely in orb-weavers</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>78</v>
-      </c>
-      <c r="D45" t="n">
-        <v>1.869858029723422</v>
-      </c>
-      <c r="E45" t="n">
-        <v>0.1957680082602067</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>0.0052</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0.9948</v>
-      </c>
-      <c r="I45" t="n">
-        <v>0.4507</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0.5493</v>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>129225023</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>GO:0007218 [Name: neuropeptide signaling pathway]</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>FMRFamide propeptide</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
           <t>myomodulin neuropeptides</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>N5.HOG0069291</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Duplication more likely in orb-weavers</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>81</v>
-      </c>
-      <c r="D46" t="n">
-        <v>-1.061098203373602</v>
-      </c>
-      <c r="E46" t="n">
-        <v>1.99174529542603</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>0.9257</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0.0743</v>
-      </c>
-      <c r="I46" t="n">
-        <v>0.0183</v>
-      </c>
-      <c r="J46" t="n">
-        <v>0.9817</v>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>129231096</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>GO:0046580 [Name: negative regulation of Ras protein signal transduction]; GO:0016020 [Name: membrane]; GO:0040037 [Name: negative regulation of fibroblast growth factor receptor signaling pathway]; GO:0005829 [Name: cytosol]; GO:0007275 [Name: multicellular organism development]; GO:0043407 [Name: negative regulation of MAP kinase activity]; GO:0048513 [Name: animal organ development]</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>sprouty signaling antagonist</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>protein sprouty</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>N5.HOG0069297</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Loss more likely in non-orb-weavers</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>68</v>
-      </c>
-      <c r="D47" t="n">
-        <v>-1.850336701795212</v>
-      </c>
-      <c r="E47" t="n">
-        <v>0.2027285561145182</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>0.966</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0.5613</v>
-      </c>
-      <c r="J47" t="n">
-        <v>0.4385</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>129217507</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>GO:0005576 [Name: extracellular region]; GO:0005615 [Name: extracellular space]; GO:0005125 [Name: cytokine activity]; GO:0030182 [Name: neuron differentiation]; GO:0005109 [Name: frizzled binding]; GO:0007275 [Name: multicellular organism development]; GO:0045165 [Name: cell fate commitment]; GO:0060070 [Name: canonical Wnt signaling pathway]</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>Wnt oncogene analog 6</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>protein Wnt-6 isoform X1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update all supp tables except intersections
</commit_message>
<xml_diff>
--- a/results/Supplementary_Table_6_OddsRatioTest_interesting_hits.xlsx
+++ b/results/Supplementary_Table_6_OddsRatioTest_interesting_hits.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -750,7 +750,7 @@
         <v>-2.850323652297765</v>
       </c>
       <c r="E6" t="n">
-        <v>2.026190682728394</v>
+        <v>2.026190682728393</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>129233658</t>
+          <t>129233408</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005515 [Name: protein binding]; GO:0005737 [Name: cytoplasm]; GO:0006468 [Name: protein phosphorylation]; GO:0030036 [Name: actin cytoskeleton organization]; GO:0005524 [Name: ATP binding]; GO:0005634 [Name: nucleus]</t>
+          <t>GO:0005737 [Name: cytoplasm]; GO:0005634 [Name: nucleus]; GO:0005524 [Name: ATP binding]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0030036 [Name: actin cytoskeleton organization]; GO:0005515 [Name: protein binding]; GO:0006468 [Name: protein phosphorylation]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1119,17 +1119,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>129220871</t>
+          <t>129226009</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>GO:0005515 [Name: protein binding]; GO:0005829 [Name: cytosol]; GO:0022008 [Name: neurogenesis]</t>
+          <t>GO:0005515 [Name: protein binding]; GO:0005829 [Name: cytosol]; GO:0022008 [Name: neurogenesis]; GO:0000932 [Name: P-body]</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>BTB/POZ domain-containing protein 6-like</t>
+          <t>BTB/POZ domain-containing protein 3-like</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1199,80 +1199,80 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>N5.HOG0034467</t>
+          <t>N5.HOG0033903</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Loss more likely in orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers, duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D14" t="n">
-        <v>1.667422234094606</v>
+        <v>-2.851770087724425</v>
       </c>
       <c r="E14" t="n">
-        <v>-1.28033039179645</v>
+        <v>2.471329191617042</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes for both tests</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.0158</v>
+        <v>0.9558</v>
       </c>
       <c r="H14" t="n">
-        <v>0.9842</v>
+        <v>0.0442</v>
       </c>
       <c r="I14" t="n">
-        <v>0.7733</v>
+        <v>0.0055</v>
       </c>
       <c r="J14" t="n">
-        <v>0.2267</v>
+        <v>0.9945000000000001</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>129230589</t>
+          <t>129223443</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>GO:0005875 [Name: microtubule associated complex]; GO:0007409 [Name: axonogenesis]; GO:0045202 [Name: synapse]; GO:0030425 [Name: dendrite]; GO:0003779 [Name: actin binding]; GO:0005829 [Name: cytosol]; GO:0005874 [Name: microtubule]; GO:0000226 [Name: microtubule cytoskeleton organization]; GO:0031114 [Name: regulation of microtubule depolymerization]; GO:0043025 [Name: neuronal cell body]; GO:0016358 [Name: dendrite development]; GO:0008017 [Name: microtubule binding]</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>microtubule-associated protein futsch-like</t>
+          <t>progranulin-like</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>microtubule-associated protein futsch</t>
+          <t>progranulin isoform X1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>N5.HOG0035629</t>
+          <t>N5.HOG0034467</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Duplication more likely in orb-weavers</t>
+          <t>Loss more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D15" t="n">
-        <v>-1.684498986055916</v>
+        <v>1.667422234094606</v>
       </c>
       <c r="E15" t="n">
-        <v>1.424655213785957</v>
+        <v>-1.28033039179645</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1280,100 +1280,100 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.9002</v>
+        <v>0.0158</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0998</v>
+        <v>0.9842</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0405</v>
+        <v>0.7733</v>
       </c>
       <c r="J15" t="n">
-        <v>0.9595</v>
+        <v>0.2267</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>129234338</t>
+          <t>129230589</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>GO:0000981 [Name: RNA polymerase II transcription factor activity, sequence-specific DNA binding]; GO:0006357 [Name: regulation of transcription from RNA polymerase II promoter]; GO:0000977 [Name: RNA polymerase II regulatory region sequence-specific DNA binding]; GO:0030182 [Name: neuron differentiation]; GO:0005634 [Name: nucleus]</t>
+          <t>GO:0005875 [Name: microtubule associated complex]; GO:0007409 [Name: axonogenesis]; GO:0045202 [Name: synapse]; GO:0030425 [Name: dendrite]; GO:0003779 [Name: actin binding]; GO:0005829 [Name: cytosol]; GO:0005874 [Name: microtubule]; GO:0000226 [Name: microtubule cytoskeleton organization]; GO:0031114 [Name: regulation of microtubule depolymerization]; GO:0043025 [Name: neuronal cell body]; GO:0016358 [Name: dendrite development]; GO:0008017 [Name: microtubule binding]</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>LIM/homeobox protein Lhx1-like</t>
+          <t>microtubule-associated protein futsch-like</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>LOW QUALITY PROTEIN: LIM/homeobox protein Lhx1</t>
+          <t>microtubule-associated protein futsch</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>N5.HOG0036003</t>
+          <t>N5.HOG0035629</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="D16" t="n">
-        <v>-3.79089242176013</v>
+        <v>-1.684498986055916</v>
       </c>
       <c r="E16" t="n">
-        <v>0.5767808481942522</v>
+        <v>1.424655213785957</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0.9523</v>
+        <v>0.9002</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0477</v>
+        <v>0.0998</v>
       </c>
       <c r="I16" t="n">
-        <v>0.4166</v>
+        <v>0.0405</v>
       </c>
       <c r="J16" t="n">
-        <v>0.5834</v>
+        <v>0.9595</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>129234391</t>
+          <t>129234338</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>GO:0006164 [Name: purine nucleotide biosynthetic process]; GO:0009156 [Name: ribonucleoside monophosphate biosynthetic process]; GO:0002189 [Name: ribose phosphate diphosphokinase complex]; GO:0005737 [Name: cytoplasm]; GO:0004749 [Name: ribose phosphate diphosphokinase activity]; GO:0006015 [Name: 5-phosphoribose 1-diphosphate biosynthetic process]; GO:0000287 [Name: magnesium ion binding]</t>
+          <t>GO:0000981 [Name: RNA polymerase II transcription factor activity, sequence-specific DNA binding]; GO:0006357 [Name: regulation of transcription from RNA polymerase II promoter]; GO:0000977 [Name: RNA polymerase II regulatory region sequence-specific DNA binding]; GO:0030182 [Name: neuron differentiation]; GO:0005634 [Name: nucleus]</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>ribose-phosphate pyrophosphokinase 2-like</t>
+          <t>LIM/homeobox protein Lhx1-like</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>ribose-phosphate pyrophosphokinase 2 isoform X2</t>
+          <t>LOW QUALITY PROTEIN: LIM/homeobox protein Lhx1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>N5.HOG0040158</t>
+          <t>N5.HOG0036003</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1382,13 +1382,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D17" t="n">
-        <v>-3.126611082576801</v>
+        <v>-3.79089242176013</v>
       </c>
       <c r="E17" t="n">
-        <v>2.889692011031725</v>
+        <v>0.5767808481942522</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1396,231 +1396,231 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.955</v>
+        <v>0.9523</v>
       </c>
       <c r="H17" t="n">
-        <v>0.045</v>
+        <v>0.0477</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1277</v>
+        <v>0.4166</v>
       </c>
       <c r="J17" t="n">
-        <v>0.8723</v>
+        <v>0.5834</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>129230758</t>
+          <t>129234391</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>GO:0006897 [Name: endocytosis]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005886 [Name: plasma membrane]; GO:0090263 [Name: positive regulation of canonical Wnt signaling pathway]; GO:0005524 [Name: ATP binding]; GO:0005634 [Name: nucleus]; GO:0007165 [Name: signal transduction]; GO:0005737 [Name: cytoplasm]; GO:0018105 [Name: peptidyl-serine phosphorylation]</t>
+          <t>GO:0006164 [Name: purine nucleotide biosynthetic process]; GO:0009156 [Name: ribonucleoside monophosphate biosynthetic process]; GO:0002189 [Name: ribose phosphate diphosphokinase complex]; GO:0005737 [Name: cytoplasm]; GO:0004749 [Name: ribose phosphate diphosphokinase activity]; GO:0006015 [Name: 5-phosphoribose 1-diphosphate biosynthetic process]; GO:0000287 [Name: magnesium ion binding]</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>casein kinase I gish</t>
+          <t>ribose-phosphate pyrophosphokinase 2-like</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>casein kinase I isoform X4</t>
+          <t>ribose-phosphate pyrophosphokinase 2 isoform X2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>N5.HOG0046893</t>
+          <t>N5.HOG0040158</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Loss more likely in orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D18" t="n">
-        <v>1.420299028263379</v>
+        <v>-3.126611082576801</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.8015196595948118</v>
+        <v>2.889692011031725</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.0443</v>
+        <v>0.955</v>
       </c>
       <c r="H18" t="n">
-        <v>0.9557</v>
+        <v>0.045</v>
       </c>
       <c r="I18" t="n">
-        <v>0.7981</v>
+        <v>0.1277</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2019</v>
+        <v>0.8723</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>129224651</t>
+          <t>129230758</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>GO:0008613 [Name: diuretic hormone activity]; GO:0001664 [Name: G-protein coupled receptor binding]; GO:0007589 [Name: body fluid secretion]; GO:0005615 [Name: extracellular space]</t>
+          <t>GO:0006897 [Name: endocytosis]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005886 [Name: plasma membrane]; GO:0090263 [Name: positive regulation of canonical Wnt signaling pathway]; GO:0005524 [Name: ATP binding]; GO:0005634 [Name: nucleus]; GO:0007165 [Name: signal transduction]; GO:0005737 [Name: cytoplasm]; GO:0018105 [Name: peptidyl-serine phosphorylation]</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>diuretic hormone class 2-like</t>
+          <t>casein kinase I gish</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>diuretic hormone class 2-like</t>
+          <t>casein kinase I isoform X4</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>N5.HOG0048186</t>
+          <t>N5.HOG0046893</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="D19" t="n">
-        <v>-1.867837837277505</v>
+        <v>1.420299028263379</v>
       </c>
       <c r="E19" t="n">
-        <v>-2.544953891852447</v>
+        <v>-0.8015196595948118</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0.7672</v>
+        <v>0.0443</v>
       </c>
       <c r="H19" t="n">
-        <v>0.2328</v>
+        <v>0.9557</v>
       </c>
       <c r="I19" t="n">
-        <v>0.9968</v>
+        <v>0.7981</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0032</v>
+        <v>0.2019</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>129218892</t>
+          <t>129224651</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>GO:0001678 [Name: cellular glucose homeostasis]; GO:0005739 [Name: mitochondrion]; GO:0006096 [Name: glycolytic process]; GO:0051156 [Name: glucose 6-phosphate metabolic process]; GO:0019158 [Name: mannokinase activity]; GO:0005829 [Name: cytosol]; GO:0008865 [Name: fructokinase activity]; GO:0004340 [Name: glucokinase activity]; GO:0005524 [Name: ATP binding]; GO:0005536 [Name: glucose binding]</t>
+          <t>GO:0008613 [Name: diuretic hormone activity]; GO:0001664 [Name: G-protein coupled receptor binding]; GO:0007589 [Name: body fluid secretion]; GO:0005615 [Name: extracellular space]</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>hexokinase-1-like</t>
+          <t>diuretic hormone class 2-like</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>hexokinase type 2</t>
+          <t>diuretic hormone class 2-like</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>N5.HOG0048441</t>
+          <t>N5.HOG0048186</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="D20" t="n">
-        <v>-1.701769774016</v>
+        <v>-1.867837837277505</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.2690227423510625</v>
+        <v>-2.544953891852447</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.9536</v>
+        <v>0.7672</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0464</v>
+        <v>0.2328</v>
       </c>
       <c r="I20" t="n">
-        <v>0.6342</v>
+        <v>0.9968</v>
       </c>
       <c r="J20" t="n">
-        <v>0.3658</v>
+        <v>0.0032</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>129219213</t>
+          <t>129218892</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>GO:0098802 [Name: plasma membrane receptor complex]; GO:0046330 [Name: positive regulation of JNK cascade]; GO:0061630 [Name: ubiquitin protein ligase activity]; GO:0043122 [Name: regulation of I-kappaB kinase/NF-kappaB signaling]; GO:0033209 [Name: tumor necrosis factor-mediated signaling pathway]; GO:0070534 [Name: protein K63-linked ubiquitination]</t>
+          <t>GO:0001678 [Name: cellular glucose homeostasis]; GO:0005739 [Name: mitochondrion]; GO:0006096 [Name: glycolytic process]; GO:0051156 [Name: glucose 6-phosphate metabolic process]; GO:0019158 [Name: mannokinase activity]; GO:0005829 [Name: cytosol]; GO:0008865 [Name: fructokinase activity]; GO:0004340 [Name: glucokinase activity]; GO:0005524 [Name: ATP binding]; GO:0005536 [Name: glucose binding]</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>E3 ubiquitin-protein ligase NRDP1 elgi</t>
+          <t>hexokinase-1-like</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>E3 ubiquitin-protein ligase NRDP1</t>
+          <t>hexokinase type 2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>N5.HOG0048897</t>
+          <t>N5.HOG0048441</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Loss more likely in orb-weavers, duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D21" t="n">
-        <v>1.528545174493033</v>
+        <v>-1.701769774016</v>
       </c>
       <c r="E21" t="n">
-        <v>-2.106825375295115</v>
+        <v>-0.2690227423510625</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1628,57 +1628,57 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0.0361</v>
+        <v>0.9536</v>
       </c>
       <c r="H21" t="n">
-        <v>0.9639</v>
+        <v>0.0464</v>
       </c>
       <c r="I21" t="n">
-        <v>0.9913</v>
+        <v>0.6342</v>
       </c>
       <c r="J21" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.3658</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>129217740</t>
+          <t>129219213</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>GO:0008277 [Name: regulation of G-protein coupled receptor protein signaling pathway]; GO:0035556 [Name: intracellular signal transduction]; GO:0007186 [Name: G-protein coupled receptor signaling pathway]</t>
+          <t>GO:0098802 [Name: plasma membrane receptor complex]; GO:0046330 [Name: positive regulation of JNK cascade]; GO:0061630 [Name: ubiquitin protein ligase activity]; GO:0043122 [Name: regulation of I-kappaB kinase/NF-kappaB signaling]; GO:0033209 [Name: tumor necrosis factor-mediated signaling pathway]; GO:0070534 [Name: protein K63-linked ubiquitination]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>regulator of G-protein signaling 7-like</t>
+          <t>E3 ubiquitin-protein ligase NRDP1 elgi</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>regulator of G-protein signaling 7 isoform X2</t>
+          <t>E3 ubiquitin-protein ligase NRDP1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>N5.HOG0050702</t>
+          <t>N5.HOG0048897</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in orb-weavers, duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>95</v>
+        <v>59</v>
       </c>
       <c r="D22" t="n">
-        <v>0.8668912516335915</v>
+        <v>1.528545174493033</v>
       </c>
       <c r="E22" t="n">
-        <v>-1.480245404596741</v>
+        <v>-2.106825375295115</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1686,57 +1686,57 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0.2156</v>
+        <v>0.0361</v>
       </c>
       <c r="H22" t="n">
-        <v>0.7843</v>
+        <v>0.9639</v>
       </c>
       <c r="I22" t="n">
-        <v>0.9888</v>
+        <v>0.9913</v>
       </c>
       <c r="J22" t="n">
-        <v>0.0112</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>129224238</t>
+          <t>129217740</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>GO:0043491 [Name: protein kinase B signaling]; GO:0005942 [Name: phosphatidylinositol 3-kinase complex]; GO:0035005 [Name: 1-phosphatidylinositol-4-phosphate 3-kinase activity]; GO:0005886 [Name: plasma membrane]; GO:0048015 [Name: phosphatidylinositol-mediated signaling]; GO:0005737 [Name: cytoplasm]; GO:0016303 [Name: 1-phosphatidylinositol-3-kinase activity]; GO:0016477 [Name: cell migration]; GO:0036092 [Name: phosphatidylinositol-3-phosphate biosynthetic process]</t>
+          <t>GO:0008277 [Name: regulation of G-protein coupled receptor protein signaling pathway]; GO:0035556 [Name: intracellular signal transduction]; GO:0007186 [Name: G-protein coupled receptor signaling pathway]</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>phosphatidylinositol 3-kinase 92E</t>
+          <t>regulator of G-protein signaling 7-like</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>phosphatidylinositol 4,5-bisphosphate 3-kinase catalytic subunit delta isoform</t>
+          <t>regulator of G-protein signaling 7 isoform X2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>N5.HOG0051572</t>
+          <t>N5.HOG0050702</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Duplication more likely in orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="D23" t="n">
-        <v>-2.647951965886426</v>
+        <v>0.8668912516335915</v>
       </c>
       <c r="E23" t="n">
-        <v>1.636211633780647</v>
+        <v>-1.480245404596741</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1744,158 +1744,158 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>0.9328</v>
+        <v>0.2156</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0672</v>
+        <v>0.7843</v>
       </c>
       <c r="I23" t="n">
-        <v>0.0365</v>
+        <v>0.9888</v>
       </c>
       <c r="J23" t="n">
-        <v>0.9635</v>
+        <v>0.0112</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>129228238</t>
+          <t>129224238</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>GO:0001726 [Name: ruffle]; GO:0004439 [Name: phosphatidylinositol-4,5-bisphosphate 5-phosphatase activity]; GO:0005737 [Name: cytoplasm]; GO:0046856 [Name: phosphatidylinositol dephosphorylation]; GO:0005886 [Name: plasma membrane]</t>
+          <t>GO:0043491 [Name: protein kinase B signaling]; GO:0005942 [Name: phosphatidylinositol 3-kinase complex]; GO:0035005 [Name: 1-phosphatidylinositol-4-phosphate 3-kinase activity]; GO:0005886 [Name: plasma membrane]; GO:0048015 [Name: phosphatidylinositol-mediated signaling]; GO:0005737 [Name: cytoplasm]; GO:0016303 [Name: 1-phosphatidylinositol-3-kinase activity]; GO:0016477 [Name: cell migration]; GO:0036092 [Name: phosphatidylinositol-3-phosphate biosynthetic process]</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>inositol polyphosphate 5-phosphatase K-like</t>
+          <t>phosphatidylinositol 3-kinase 92E</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>phosphatidylinositol 4,5-bisphosphate 5-phosphatase A isoform X4</t>
+          <t>phosphatidylinositol 4,5-bisphosphate 3-kinase catalytic subunit delta isoform</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>N5.HOG0053555</t>
+          <t>N5.HOG0051572</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers, duplication more likely in non-orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="D24" t="n">
-        <v>-3.03255284649051</v>
+        <v>-2.647951965886426</v>
       </c>
       <c r="E24" t="n">
-        <v>-1.696958693304238</v>
+        <v>1.636211633780647</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Yes for loss; no for duplication</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>0.9943</v>
+        <v>0.9328</v>
       </c>
       <c r="H24" t="n">
-        <v>0.0057</v>
+        <v>0.0672</v>
       </c>
       <c r="I24" t="n">
-        <v>0.9959</v>
+        <v>0.0365</v>
       </c>
       <c r="J24" t="n">
-        <v>0.0041</v>
+        <v>0.9635</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>129228121</t>
+          <t>129228238</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>GO:0004749 [Name: ribose phosphate diphosphokinase activity]; GO:0006015 [Name: 5-phosphoribose 1-diphosphate biosynthetic process]; GO:0005737 [Name: cytoplasm]; GO:0006164 [Name: purine nucleotide biosynthetic process]; GO:0000287 [Name: magnesium ion binding]; GO:0002189 [Name: ribose phosphate diphosphokinase complex]</t>
+          <t>GO:0001726 [Name: ruffle]; GO:0004439 [Name: phosphatidylinositol-4,5-bisphosphate 5-phosphatase activity]; GO:0005737 [Name: cytoplasm]; GO:0046856 [Name: phosphatidylinositol dephosphorylation]; GO:0005886 [Name: plasma membrane]</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>phosphoribosyl pyrophosphate synthase-associated protein 2-like</t>
+          <t>inositol polyphosphate 5-phosphatase K-like</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>phosphoribosyl pyrophosphate synthase-associated protein 2</t>
+          <t>phosphatidylinositol 4,5-bisphosphate 5-phosphatase A isoform X4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>N5.HOG0054227</t>
+          <t>N5.HOG0053555</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers, duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="D25" t="n">
-        <v>0.3349693480177507</v>
+        <v>-3.03255284649051</v>
       </c>
       <c r="E25" t="n">
-        <v>-1.425149241466285</v>
+        <v>-1.696958693304238</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes for loss; no for duplication</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0.2231</v>
+        <v>0.9943</v>
       </c>
       <c r="H25" t="n">
-        <v>0.7768</v>
+        <v>0.0057</v>
       </c>
       <c r="I25" t="n">
-        <v>0.9701</v>
+        <v>0.9959</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0299</v>
+        <v>0.0041</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>129224230</t>
+          <t>129228121</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>GO:0035091 [Name: phosphatidylinositol binding]; GO:0008270 [Name: zinc ion binding]; GO:0003676 [Name: nucleic acid binding]</t>
+          <t>GO:0004749 [Name: ribose phosphate diphosphokinase activity]; GO:0006015 [Name: 5-phosphoribose 1-diphosphate biosynthetic process]; GO:0005737 [Name: cytoplasm]; GO:0006164 [Name: purine nucleotide biosynthetic process]; GO:0000287 [Name: magnesium ion binding]; GO:0002189 [Name: ribose phosphate diphosphokinase complex]</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>zinc finger CCHC domain-containing protein 2-like</t>
+          <t>phosphoribosyl pyrophosphate synthase-associated protein 2-like</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>zinc finger CCHC domain-containing protein 2 isoform X2</t>
+          <t>phosphoribosyl pyrophosphate synthase-associated protein 2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>N5.HOG0054901</t>
+          <t>N5.HOG0054227</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1904,13 +1904,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D26" t="n">
-        <v>-1.25678417448257</v>
+        <v>0.3349693480177507</v>
       </c>
       <c r="E26" t="n">
-        <v>-2.075131227901787</v>
+        <v>-1.425149241466285</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1918,57 +1918,57 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0.7378</v>
+        <v>0.2231</v>
       </c>
       <c r="H26" t="n">
-        <v>0.2621</v>
+        <v>0.7768</v>
       </c>
       <c r="I26" t="n">
-        <v>0.9696</v>
+        <v>0.9701</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0304</v>
+        <v>0.0299</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>129227017</t>
+          <t>129224230</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>GO:0007165 [Name: signal transduction]; GO:0005737 [Name: cytoplasm]; GO:0005634 [Name: nucleus]; GO:0018105 [Name: peptidyl-serine phosphorylation]; GO:0006897 [Name: endocytosis]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005524 [Name: ATP binding]</t>
+          <t>GO:0035091 [Name: phosphatidylinositol binding]; GO:0008270 [Name: zinc ion binding]; GO:0003676 [Name: nucleic acid binding]</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>casein kinase I-like</t>
+          <t>zinc finger CCHC domain-containing protein 2-like</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>casein kinase I</t>
+          <t>zinc finger CCHC domain-containing protein 2 isoform X2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>N5.HOG0058078</t>
+          <t>N5.HOG0054901</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Duplication more likely in orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.7256542955276075</v>
+        <v>-1.25678417448257</v>
       </c>
       <c r="E27" t="n">
-        <v>1.811869176606395</v>
+        <v>-2.075131227901787</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1976,42 +1976,42 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>0.5648</v>
+        <v>0.7378</v>
       </c>
       <c r="H27" t="n">
-        <v>0.4352</v>
+        <v>0.2621</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0498</v>
+        <v>0.9696</v>
       </c>
       <c r="J27" t="n">
-        <v>0.9502</v>
+        <v>0.0304</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>129225594</t>
+          <t>129227017</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>GO:0030425 [Name: dendrite]; GO:0048168 [Name: regulation of neuronal synaptic plasticity]; GO:0031175 [Name: neuron projection development]</t>
+          <t>GO:0007165 [Name: signal transduction]; GO:0005737 [Name: cytoplasm]; GO:0005634 [Name: nucleus]; GO:0018105 [Name: peptidyl-serine phosphorylation]; GO:0006897 [Name: endocytosis]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0005524 [Name: ATP binding]</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>neurochondrin homolog</t>
+          <t>casein kinase I-like</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>neurochondrin homolog</t>
+          <t>casein kinase I</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>N5.HOG0058262</t>
+          <t>N5.HOG0058078</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2020,13 +2020,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="D28" t="n">
-        <v>-3.486151905508599</v>
+        <v>-0.7256542955276075</v>
       </c>
       <c r="E28" t="n">
-        <v>1.530248754206848</v>
+        <v>1.811869176606395</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -2034,100 +2034,100 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0.8943</v>
+        <v>0.5648</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1057</v>
+        <v>0.4352</v>
       </c>
       <c r="I28" t="n">
-        <v>0.0228</v>
+        <v>0.0498</v>
       </c>
       <c r="J28" t="n">
-        <v>0.9772</v>
+        <v>0.9502</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>129215997</t>
+          <t>129225594</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>GO:0006470 [Name: protein dephosphorylation]; GO:0043169 [Name: cation binding]; GO:0004722 [Name: protein serine/threonine phosphatase activity]</t>
+          <t>GO:0030425 [Name: dendrite]; GO:0048168 [Name: regulation of neuronal synaptic plasticity]; GO:0031175 [Name: neuron projection development]</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>TGF-beta-activated kinase 1 and MAP3K7-binding protein 1-like</t>
+          <t>neurochondrin homolog</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>TGF-beta-activated kinase 1 and MAP3K7-binding protein 1 isoform X1</t>
+          <t>neurochondrin homolog</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>N5.HOG0059968</t>
+          <t>N5.HOG0058262</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in orb-weavers</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D29" t="n">
-        <v>-3.96907534691269</v>
+        <v>-3.486151905508599</v>
       </c>
       <c r="E29" t="n">
-        <v>0.1487060270050904</v>
+        <v>1.530248754206848</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>0.9863</v>
+        <v>0.8943</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0137</v>
+        <v>0.1057</v>
       </c>
       <c r="I29" t="n">
-        <v>0.3737</v>
+        <v>0.0228</v>
       </c>
       <c r="J29" t="n">
-        <v>0.6263</v>
+        <v>0.9772</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>129224556</t>
+          <t>129215997</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>GO:0005886 [Name: plasma membrane]; GO:0046854 [Name: phosphatidylinositol phosphorylation]; GO:0072659 [Name: protein localization to plasma membrane]</t>
+          <t>GO:0006470 [Name: protein dephosphorylation]; GO:0043169 [Name: cation binding]; GO:0004722 [Name: protein serine/threonine phosphatase activity]</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>PI4KA lipid kinase complex subunit hyccin</t>
+          <t>TGF-beta-activated kinase 1 and MAP3K7-binding protein 1-like</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>hyccin</t>
+          <t>TGF-beta-activated kinase 1 and MAP3K7-binding protein 1 isoform X1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>N5.HOG0060288</t>
+          <t>N5.HOG0059968</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2136,71 +2136,71 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="D30" t="n">
-        <v>-2.702517333918679</v>
+        <v>-3.96907534691269</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.487062078600888</v>
+        <v>0.1487060270050904</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0.9528</v>
+        <v>0.9863</v>
       </c>
       <c r="H30" t="n">
-        <v>0.0472</v>
+        <v>0.0137</v>
       </c>
       <c r="I30" t="n">
-        <v>0.5478</v>
+        <v>0.3737</v>
       </c>
       <c r="J30" t="n">
-        <v>0.4522</v>
+        <v>0.6263</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>129222137</t>
+          <t>129224556</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>GO:0005634 [Name: nucleus]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0044773 [Name: mitotic DNA damage checkpoint]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]</t>
+          <t>GO:0005886 [Name: plasma membrane]; GO:0046854 [Name: phosphatidylinositol phosphorylation]; GO:0072659 [Name: protein localization to plasma membrane]</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>cell division cycle 7-related protein kinase-like</t>
+          <t>PI4KA lipid kinase complex subunit hyccin</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>cell division cycle 7-related protein kinase isoform X1</t>
+          <t>hyccin</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>N5.HOG0061119</t>
+          <t>N5.HOG0060288</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="D31" t="n">
-        <v>1.071261968122538</v>
+        <v>-2.702517333918679</v>
       </c>
       <c r="E31" t="n">
-        <v>-2.054862693041546</v>
+        <v>-0.487062078600888</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -2208,42 +2208,42 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>0.1148</v>
+        <v>0.9528</v>
       </c>
       <c r="H31" t="n">
-        <v>0.8852</v>
+        <v>0.0472</v>
       </c>
       <c r="I31" t="n">
-        <v>0.9719</v>
+        <v>0.5478</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0281</v>
+        <v>0.4522</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>129225556</t>
+          <t>129222137</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>GO:0006811 [Name: ion transport]; GO:0043005 [Name: neuron projection]; GO:0035235 [Name: ionotropic glutamate receptor signaling pathway]; GO:0042391 [Name: regulation of membrane potential]; GO:0005886 [Name: plasma membrane]; GO:0017146 [Name: NMDA selective glutamate receptor complex]; GO:0045202 [Name: synapse]; GO:0004972 [Name: NMDA glutamate receptor activity]; GO:0007268 [Name: chemical synaptic transmission]</t>
+          <t>GO:0005634 [Name: nucleus]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0044773 [Name: mitotic DNA damage checkpoint]; GO:0006468 [Name: protein phosphorylation]; GO:0005524 [Name: ATP binding]</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>glutamate [NMDA] receptor subunit 1-like</t>
+          <t>cell division cycle 7-related protein kinase-like</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>glutamate [NMDA</t>
+          <t>cell division cycle 7-related protein kinase isoform X1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>N5.HOG0061199</t>
+          <t>N5.HOG0061119</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2252,13 +2252,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.7254076171249628</v>
+        <v>1.071261968122538</v>
       </c>
       <c r="E32" t="n">
-        <v>-2.022475220611714</v>
+        <v>-2.054862693041546</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -2266,42 +2266,42 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>0.5127</v>
+        <v>0.1148</v>
       </c>
       <c r="H32" t="n">
-        <v>0.4873</v>
+        <v>0.8852</v>
       </c>
       <c r="I32" t="n">
-        <v>0.9658</v>
+        <v>0.9719</v>
       </c>
       <c r="J32" t="n">
-        <v>0.0342</v>
+        <v>0.0281</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>129227869</t>
+          <t>129225556</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>GO:0046579 [Name: positive regulation of Ras protein signal transduction]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0006468 [Name: protein phosphorylation]</t>
+          <t>GO:0006811 [Name: ion transport]; GO:0043005 [Name: neuron projection]; GO:0035235 [Name: ionotropic glutamate receptor signaling pathway]; GO:0042391 [Name: regulation of membrane potential]; GO:0005886 [Name: plasma membrane]; GO:0017146 [Name: NMDA selective glutamate receptor complex]; GO:0045202 [Name: synapse]; GO:0004972 [Name: NMDA glutamate receptor activity]; GO:0007268 [Name: chemical synaptic transmission]</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>serine/threonine-protein kinase 19-like</t>
+          <t>glutamate [NMDA] receptor subunit 1-like</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>inactive serine/threonine-protein kinase 19</t>
+          <t>glutamate [NMDA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>N5.HOG0062578</t>
+          <t>N5.HOG0061199</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2310,56 +2310,56 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D33" t="n">
-        <v>0.3349693480177507</v>
+        <v>-0.7254076171249628</v>
       </c>
       <c r="E33" t="n">
-        <v>-2.369802435297485</v>
+        <v>-2.022475220611714</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>0.2231</v>
+        <v>0.5127</v>
       </c>
       <c r="H33" t="n">
-        <v>0.7768</v>
+        <v>0.4873</v>
       </c>
       <c r="I33" t="n">
-        <v>0.9826</v>
+        <v>0.9658</v>
       </c>
       <c r="J33" t="n">
-        <v>0.0174</v>
+        <v>0.0342</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>129216091</t>
+          <t>129227869</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>GO:0019543 [Name: propionate catabolic process]; GO:0005829 [Name: cytosol]; GO:0004613 [Name: phosphoenolpyruvate carboxykinase (GTP) activity]; GO:0005525 [Name: GTP binding]; GO:0046327 [Name: glycerol biosynthetic process from pyruvate]; GO:0006094 [Name: gluconeogenesis]; GO:0030145 [Name: manganese ion binding]; GO:0032869 [Name: cellular response to insulin stimulus]; GO:0042594 [Name: response to starvation]; GO:0070365 [Name: hepatocyte differentiation]; GO:0071333 [Name: cellular response to glucose stimulus]; GO:0071549 [Name: cellular response to dexamethasone stimulus]</t>
+          <t>GO:0046579 [Name: positive regulation of Ras protein signal transduction]; GO:0004674 [Name: protein serine/threonine kinase activity]; GO:0006468 [Name: protein phosphorylation]</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>phosphoenolpyruvate carboxykinase, cytosolic [GTP]-like</t>
+          <t>serine/threonine-protein kinase 19-like</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>phosphoenolpyruvate carboxykinase, cytosolic [GTP</t>
+          <t>inactive serine/threonine-protein kinase 19</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>N5.HOG0063077</t>
+          <t>N5.HOG0062578</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2368,71 +2368,71 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D34" t="n">
-        <v>-1.260837948086103</v>
+        <v>0.3349693480177507</v>
       </c>
       <c r="E34" t="n">
-        <v>-1.784817696803436</v>
+        <v>-2.369802435297485</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>0.7608</v>
+        <v>0.2231</v>
       </c>
       <c r="H34" t="n">
-        <v>0.2392</v>
+        <v>0.7768</v>
       </c>
       <c r="I34" t="n">
-        <v>0.9733000000000001</v>
+        <v>0.9826</v>
       </c>
       <c r="J34" t="n">
-        <v>0.0267</v>
+        <v>0.0174</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>129219268</t>
+          <t>129216091</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>GO:0043025 [Name: neuronal cell body]; GO:0045727 [Name: positive regulation of translation]; GO:0043197 [Name: dendritic spine]; GO:0048814 [Name: regulation of dendrite morphogenesis]; GO:0016020 [Name: membrane]; GO:0071598 [Name: neuronal ribonucleoprotein granule]; GO:0003730 [Name: mRNA 3'-UTR binding]; GO:0030424 [Name: axon]; GO:0042803 [Name: protein homodimerization activity]; GO:0043488 [Name: regulation of mRNA stability]; GO:0060998 [Name: regulation of dendritic spine development]; GO:0099578 [Name: regulation of translation at postsynapse, modulating synaptic transmission]; GO:0008089 [Name: anterograde axonal transport]; GO:0014069 [Name: postsynaptic density]; GO:0045182 [Name: translation regulator activity]; GO:0005634 [Name: nucleus]; GO:0007417 [Name: central nervous system development]; GO:0017148 [Name: negative regulation of translation]; GO:1905244 [Name: regulation of modification of synaptic structure]</t>
+          <t>GO:0019543 [Name: propionate catabolic process]; GO:0005829 [Name: cytosol]; GO:0004613 [Name: phosphoenolpyruvate carboxykinase (GTP) activity]; GO:0005525 [Name: GTP binding]; GO:0046327 [Name: glycerol biosynthetic process from pyruvate]; GO:0006094 [Name: gluconeogenesis]; GO:0030145 [Name: manganese ion binding]; GO:0032869 [Name: cellular response to insulin stimulus]; GO:0042594 [Name: response to starvation]; GO:0070365 [Name: hepatocyte differentiation]; GO:0071333 [Name: cellular response to glucose stimulus]; GO:0071549 [Name: cellular response to dexamethasone stimulus]</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>fragile X messenger ribonucleoprotein 1 homolog</t>
+          <t>phosphoenolpyruvate carboxykinase, cytosolic [GTP]-like</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>RNA-binding protein FXR1</t>
+          <t>phosphoenolpyruvate carboxykinase, cytosolic [GTP</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>N5.HOG0066939</t>
+          <t>N5.HOG0063077</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69</v>
+        <v>96</v>
       </c>
       <c r="D35" t="n">
-        <v>-2.650703581186066</v>
+        <v>-1.260837948086103</v>
       </c>
       <c r="E35" t="n">
-        <v>0.939259027269308</v>
+        <v>-1.784817696803436</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2440,209 +2440,383 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>0.9714</v>
+        <v>0.7608</v>
       </c>
       <c r="H35" t="n">
-        <v>0.0286</v>
+        <v>0.2392</v>
       </c>
       <c r="I35" t="n">
-        <v>0.0699</v>
+        <v>0.9733000000000001</v>
       </c>
       <c r="J35" t="n">
-        <v>0.9301</v>
+        <v>0.0267</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>129228009</t>
+          <t>129219268</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>GO:0015250 [Name: water channel activity]; GO:0055085 [Name: transmembrane transport]; GO:0005886 [Name: plasma membrane]</t>
+          <t>GO:0043025 [Name: neuronal cell body]; GO:0045727 [Name: positive regulation of translation]; GO:0043197 [Name: dendritic spine]; GO:0048814 [Name: regulation of dendrite morphogenesis]; GO:0016020 [Name: membrane]; GO:0071598 [Name: neuronal ribonucleoprotein granule]; GO:0003730 [Name: mRNA 3'-UTR binding]; GO:0030424 [Name: axon]; GO:0042803 [Name: protein homodimerization activity]; GO:0043488 [Name: regulation of mRNA stability]; GO:0060998 [Name: regulation of dendritic spine development]; GO:0099578 [Name: regulation of translation at postsynapse, modulating synaptic transmission]; GO:0008089 [Name: anterograde axonal transport]; GO:0014069 [Name: postsynaptic density]; GO:0045182 [Name: translation regulator activity]; GO:0005634 [Name: nucleus]; GO:0007417 [Name: central nervous system development]; GO:0017148 [Name: negative regulation of translation]; GO:1905244 [Name: regulation of modification of synaptic structure]</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>neurogenic protein big brain-like</t>
+          <t>fragile X messenger ribonucleoprotein 1 homolog</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>aquaporin AQPAe.a</t>
+          <t>RNA-binding protein FXR1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>N5.HOG0067099</t>
+          <t>N5.HOG0066939</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Duplication more likely in non-orb-weavers</t>
+          <t>Loss more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="D36" t="n">
-        <v>2.257461790658672</v>
+        <v>-2.650703581186066</v>
       </c>
       <c r="E36" t="n">
-        <v>-2.780945563596604</v>
+        <v>0.939259027269308</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>0.083</v>
+        <v>0.9714</v>
       </c>
       <c r="H36" t="n">
-        <v>0.917</v>
+        <v>0.0286</v>
       </c>
       <c r="I36" t="n">
-        <v>0.9689</v>
+        <v>0.0699</v>
       </c>
       <c r="J36" t="n">
-        <v>0.0311</v>
+        <v>0.9301</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>129225034</t>
+          <t>129228009</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>GO:0005737 [Name: cytoplasm]; GO:0019901 [Name: protein kinase binding]; GO:0045737 [Name: positive regulation of cyclin-dependent protein serine/threonine kinase activity]; GO:0061575 [Name: cyclin-dependent protein serine/threonine kinase activator activity]; GO:0032147 [Name: activation of protein kinase activity]; GO:0016533 [Name: cyclin-dependent protein kinase 5 holoenzyme complex]</t>
+          <t>GO:0015250 [Name: water channel activity]; GO:0055085 [Name: transmembrane transport]; GO:0005886 [Name: plasma membrane]</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Cdk5 activator-like protein</t>
+          <t>neurogenic protein big brain-like</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>cyclin-dependent kinase 5 activator 1 isoform X1</t>
+          <t>aquaporin AQPAe.a</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>N5.HOG0068715</t>
+          <t>N5.HOG0067099</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Loss more likely in non-orb-weavers</t>
+          <t>Duplication more likely in non-orb-weavers</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="D37" t="n">
-        <v>-2.162736198321358</v>
+        <v>2.257461790658672</v>
       </c>
       <c r="E37" t="n">
-        <v>0.7122931788181197</v>
+        <v>-2.780945563596604</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>0.991</v>
+        <v>0.083</v>
       </c>
       <c r="H37" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.917</v>
       </c>
       <c r="I37" t="n">
-        <v>0.2442</v>
+        <v>0.9689</v>
       </c>
       <c r="J37" t="n">
-        <v>0.7558</v>
+        <v>0.0311</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>129232140</t>
+          <t>129225034</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>GO:0004930 [Name: G-protein coupled receptor activity]; GO:0007186 [Name: G-protein coupled receptor signaling pathway]; GO:0016020 [Name: membrane]</t>
+          <t>GO:0005737 [Name: cytoplasm]; GO:0019901 [Name: protein kinase binding]; GO:0045737 [Name: positive regulation of cyclin-dependent protein serine/threonine kinase activity]; GO:0061575 [Name: cyclin-dependent protein serine/threonine kinase activator activity]; GO:0032147 [Name: activation of protein kinase activity]; GO:0016533 [Name: cyclin-dependent protein kinase 5 holoenzyme complex]</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>probable G-protein coupled receptor AH9.1</t>
+          <t>Cdk5 activator-like protein</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>probable G-protein coupled receptor AH9.1</t>
+          <t>cyclin-dependent kinase 5 activator 1 isoform X1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>N5.HOG0067221</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Duplication more likely in orb-weavers</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>89</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-1.50443128599423</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1.649683623026397</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>0.9095</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.0905</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.9787</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>129222939</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>GO:0006670 [Name: sphingosine metabolic process]; GO:0046839 [Name: phospholipid dephosphorylation]; GO:0042392 [Name: sphingosine-1-phosphate phosphatase activity]; GO:0005789 [Name: endoplasmic reticulum membrane]</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>sphingosine-1-phosphate phosphatase 2-like</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>sphingosine-1-phosphate phosphatase 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>N5.HOG0068715</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Loss more likely in non-orb-weavers</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>83</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-2.162736198321358</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.7122931788181197</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.2442</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.7558</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>129232140</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>GO:0004930 [Name: G-protein coupled receptor activity]; GO:0007186 [Name: G-protein coupled receptor signaling pathway]; GO:0016020 [Name: membrane]</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>probable G-protein coupled receptor AH9.1</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>probable G-protein coupled receptor AH9.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>N5.HOG0068937</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Loss more likely in orb-weavers</t>
         </is>
       </c>
-      <c r="C38" t="n">
+      <c r="C40" t="n">
         <v>78</v>
       </c>
-      <c r="D38" t="n">
+      <c r="D40" t="n">
         <v>1.716305137494582</v>
       </c>
-      <c r="E38" t="n">
+      <c r="E40" t="n">
         <v>-0.2263921591536401</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G38" t="n">
+      <c r="G40" t="n">
         <v>0.0063</v>
       </c>
-      <c r="H38" t="n">
+      <c r="H40" t="n">
         <v>0.9937</v>
       </c>
-      <c r="I38" t="n">
+      <c r="I40" t="n">
         <v>0.5667</v>
       </c>
-      <c r="J38" t="n">
+      <c r="J40" t="n">
         <v>0.4333</v>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>129225023</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>GO:0007218 [Name: neuropeptide signaling pathway]</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>FMRFamide propeptide</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>myomodulin neuropeptides</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>N5.HOG0069577</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Loss more likely in non-orb-weavers</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>81</v>
+      </c>
+      <c r="D41" t="n">
+        <v>-1.740438071842964</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.3524636238108737</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>0.9532</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.2143</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.7857</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>129219120</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>GO:0000981 [Name: RNA polymerase II transcription factor activity, sequence-specific DNA binding]; GO:0005634 [Name: nucleus]; GO:0006357 [Name: regulation of transcription from RNA polymerase II promoter]; GO:0030154 [Name: cell differentiation]; GO:0000978 [Name: RNA polymerase II core promoter proximal region sequence-specific DNA binding]</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>homeobox protein vnd-like</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>homeobox protein Nkx-2.5</t>
         </is>
       </c>
     </row>

</xml_diff>